<commit_message>
Fix N/A errors in Eliminatorias and use safe columns insertion
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_Final_vacia.xlsx
+++ b/Quiniela_Mundial_2026_Final_vacia.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -141,8 +141,11 @@
       <color rgb="00333333"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -197,8 +200,14 @@
         <bgColor rgb="00F8D7DA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEEEEE"/>
+        <bgColor rgb="00EEEEEE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -257,12 +266,26 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -357,6 +380,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="9" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -6125,11 +6151,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="16" min="2" max="2"/>
-    <col width="20" customWidth="1" style="16" min="6" max="7"/>
+    <col width="6" customWidth="1" style="16" min="3" max="3"/>
+    <col width="6" customWidth="1" style="16" min="4" max="4"/>
+    <col width="3" customWidth="1" style="16" min="5" max="5"/>
+    <col width="6" customWidth="1" style="16" min="6" max="7"/>
+    <col width="6" customWidth="1" style="16" min="7" max="7"/>
+    <col width="18" customWidth="1" style="16" min="8" max="8"/>
+    <col width="18" customWidth="1" style="16" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6163,29 +6195,34 @@
           <t>Goles</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Pen.</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
         <is>
           <t>vs</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Pen.</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
         <is>
           <t>Goles</t>
         </is>
       </c>
-      <c r="F5" s="14" t="inlineStr">
+      <c r="H5" s="14" t="inlineStr">
         <is>
           <t>Equipo B</t>
         </is>
       </c>
-      <c r="G5" s="14" t="inlineStr">
+      <c r="I5" s="14" t="inlineStr">
         <is>
           <t>Clasifica</t>
-        </is>
-      </c>
-      <c r="H5" s="14" t="inlineStr">
-        <is>
-          <t>Estado</t>
         </is>
       </c>
     </row>
@@ -6200,18 +6237,20 @@
         <v/>
       </c>
       <c r="C6" s="5" t="n"/>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="38" t="n"/>
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6">
+      <c r="F6" s="38" t="n"/>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6">
         <f>Backend!C3</f>
         <v/>
       </c>
-      <c r="G6">
-        <f>IF(AND(ISNUMBER(C6),ISNUMBER(E6)),IF(C6&gt;E6,B6,F6),"")</f>
+      <c r="I6">
+        <f>IF(OR(C6="", G6=""), "", IF(C6&gt;G6, B6, IF(G6&gt;C6, H6, IF(D6&gt;F6, B6, IF(F6&gt;D6, H6, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6226,18 +6265,20 @@
         <v/>
       </c>
       <c r="C7" s="5" t="n"/>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="38" t="n"/>
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7">
+      <c r="F7" s="38" t="n"/>
+      <c r="G7" s="5" t="n"/>
+      <c r="H7">
         <f>Backend!C4</f>
         <v/>
       </c>
-      <c r="G7">
-        <f>IF(AND(ISNUMBER(C7),ISNUMBER(E7)),IF(C7&gt;E7,B7,F7),"")</f>
+      <c r="I7">
+        <f>IF(OR(C7="", G7=""), "", IF(C7&gt;G7, B7, IF(G7&gt;C7, H7, IF(D7&gt;F7, B7, IF(F7&gt;D7, H7, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6252,18 +6293,20 @@
         <v/>
       </c>
       <c r="C8" s="5" t="n"/>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="38" t="n"/>
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8">
-        <f>INDEX(Backend!$C$16:$C$23, MATCH(VLOOKUP(Backend!$D$29, MatrizTerceros!$A$1:$I$495, 5, FALSE), Backend!$B$16:$B$23, 0))</f>
-        <v/>
-      </c>
-      <c r="G8">
-        <f>IF(AND(ISNUMBER(C8),ISNUMBER(E8)),IF(C8&gt;E8,B8,F8),"")</f>
+      <c r="F8" s="38" t="n"/>
+      <c r="G8" s="5" t="n"/>
+      <c r="H8">
+        <f>IFERROR(INDEX(Backend!$C$16:$C$23, MATCH(VLOOKUP(Backend!$D$29, MatrizTerceros!$A$1:$I$495, 5, FALSE), Backend!$B$16:$B$23, 0)), "")</f>
+        <v/>
+      </c>
+      <c r="I8">
+        <f>IF(OR(C8="", G8=""), "", IF(C8&gt;G8, B8, IF(G8&gt;C8, H8, IF(D8&gt;F8, B8, IF(F8&gt;D8, H8, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6278,18 +6321,20 @@
         <v/>
       </c>
       <c r="C9" s="5" t="n"/>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="38" t="n"/>
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9">
-        <f>INDEX(Backend!$C$16:$C$23, MATCH(VLOOKUP(Backend!$D$29, MatrizTerceros!$A$1:$I$495, 7, FALSE), Backend!$B$16:$B$23, 0))</f>
-        <v/>
-      </c>
-      <c r="G9">
-        <f>IF(AND(ISNUMBER(C9),ISNUMBER(E9)),IF(C9&gt;E9,B9,F9),"")</f>
+      <c r="F9" s="38" t="n"/>
+      <c r="G9" s="5" t="n"/>
+      <c r="H9">
+        <f>IFERROR(INDEX(Backend!$C$16:$C$23, MATCH(VLOOKUP(Backend!$D$29, MatrizTerceros!$A$1:$I$495, 7, FALSE), Backend!$B$16:$B$23, 0)), "")</f>
+        <v/>
+      </c>
+      <c r="I9">
+        <f>IF(OR(C9="", G9=""), "", IF(C9&gt;G9, B9, IF(G9&gt;C9, H9, IF(D9&gt;F9, B9, IF(F9&gt;D9, H9, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6304,18 +6349,20 @@
         <v/>
       </c>
       <c r="C10" s="5" t="n"/>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="38" t="n"/>
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10">
+      <c r="F10" s="38" t="n"/>
+      <c r="G10" s="5" t="n"/>
+      <c r="H10">
         <f>Backend!C7</f>
         <v/>
       </c>
-      <c r="G10">
-        <f>IF(AND(ISNUMBER(C10),ISNUMBER(E10)),IF(C10&gt;E10,B10,F10),"")</f>
+      <c r="I10">
+        <f>IF(OR(C10="", G10=""), "", IF(C10&gt;G10, B10, IF(G10&gt;C10, H10, IF(D10&gt;F10, B10, IF(F10&gt;D10, H10, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6330,18 +6377,20 @@
         <v/>
       </c>
       <c r="C11" s="5" t="n"/>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="38" t="n"/>
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11">
+      <c r="F11" s="38" t="n"/>
+      <c r="G11" s="5" t="n"/>
+      <c r="H11">
         <f>Backend!C10</f>
         <v/>
       </c>
-      <c r="G11">
-        <f>IF(AND(ISNUMBER(C11),ISNUMBER(E11)),IF(C11&gt;E11,B11,F11),"")</f>
+      <c r="I11">
+        <f>IF(OR(C11="", G11=""), "", IF(C11&gt;G11, B11, IF(G11&gt;C11, H11, IF(D11&gt;F11, B11, IF(F11&gt;D11, H11, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6356,18 +6405,20 @@
         <v/>
       </c>
       <c r="C12" s="5" t="n"/>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D12" s="38" t="n"/>
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12">
-        <f>INDEX(Backend!$C$16:$C$23, MATCH(VLOOKUP(Backend!$D$29, MatrizTerceros!$A$1:$I$495, 2, FALSE), Backend!$B$16:$B$23, 0))</f>
-        <v/>
-      </c>
-      <c r="G12">
-        <f>IF(AND(ISNUMBER(C12),ISNUMBER(E12)),IF(C12&gt;E12,B12,F12),"")</f>
+      <c r="F12" s="38" t="n"/>
+      <c r="G12" s="5" t="n"/>
+      <c r="H12">
+        <f>IFERROR(INDEX(Backend!$C$16:$C$23, MATCH(VLOOKUP(Backend!$D$29, MatrizTerceros!$A$1:$I$495, 2, FALSE), Backend!$B$16:$B$23, 0)), "")</f>
+        <v/>
+      </c>
+      <c r="I12">
+        <f>IF(OR(C12="", G12=""), "", IF(C12&gt;G12, B12, IF(G12&gt;C12, H12, IF(D12&gt;F12, B12, IF(F12&gt;D12, H12, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6382,18 +6433,20 @@
         <v/>
       </c>
       <c r="C13" s="5" t="n"/>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D13" s="38" t="n"/>
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13">
-        <f>INDEX(Backend!$C$16:$C$23, MATCH(VLOOKUP(Backend!$D$29, MatrizTerceros!$A$1:$I$495, 9, FALSE), Backend!$B$16:$B$23, 0))</f>
-        <v/>
-      </c>
-      <c r="G13">
-        <f>IF(AND(ISNUMBER(C13),ISNUMBER(E13)),IF(C13&gt;E13,B13,F13),"")</f>
+      <c r="F13" s="38" t="n"/>
+      <c r="G13" s="5" t="n"/>
+      <c r="H13">
+        <f>IFERROR(INDEX(Backend!$C$16:$C$23, MATCH(VLOOKUP(Backend!$D$29, MatrizTerceros!$A$1:$I$495, 9, FALSE), Backend!$B$16:$B$23, 0)), "")</f>
+        <v/>
+      </c>
+      <c r="I13">
+        <f>IF(OR(C13="", G13=""), "", IF(C13&gt;G13, B13, IF(G13&gt;C13, H13, IF(D13&gt;F13, B13, IF(F13&gt;D13, H13, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6408,18 +6461,20 @@
         <v/>
       </c>
       <c r="C14" s="5" t="n"/>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D14" s="38" t="n"/>
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14">
-        <f>INDEX(Backend!$C$16:$C$23, MATCH(VLOOKUP(Backend!$D$29, MatrizTerceros!$A$1:$I$495, 4, FALSE), Backend!$B$16:$B$23, 0))</f>
-        <v/>
-      </c>
-      <c r="G14">
-        <f>IF(AND(ISNUMBER(C14),ISNUMBER(E14)),IF(C14&gt;E14,B14,F14),"")</f>
+      <c r="F14" s="38" t="n"/>
+      <c r="G14" s="5" t="n"/>
+      <c r="H14">
+        <f>IFERROR(INDEX(Backend!$C$16:$C$23, MATCH(VLOOKUP(Backend!$D$29, MatrizTerceros!$A$1:$I$495, 4, FALSE), Backend!$B$16:$B$23, 0)), "")</f>
+        <v/>
+      </c>
+      <c r="I14">
+        <f>IF(OR(C14="", G14=""), "", IF(C14&gt;G14, B14, IF(G14&gt;C14, H14, IF(D14&gt;F14, B14, IF(F14&gt;D14, H14, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6434,18 +6489,20 @@
         <v/>
       </c>
       <c r="C15" s="5" t="n"/>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D15" s="38" t="n"/>
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15">
-        <f>INDEX(Backend!$C$16:$C$23, MATCH(VLOOKUP(Backend!$D$29, MatrizTerceros!$A$1:$I$495, 6, FALSE), Backend!$B$16:$B$23, 0))</f>
-        <v/>
-      </c>
-      <c r="G15">
-        <f>IF(AND(ISNUMBER(C15),ISNUMBER(E15)),IF(C15&gt;E15,B15,F15),"")</f>
+      <c r="F15" s="38" t="n"/>
+      <c r="G15" s="5" t="n"/>
+      <c r="H15">
+        <f>IFERROR(INDEX(Backend!$C$16:$C$23, MATCH(VLOOKUP(Backend!$D$29, MatrizTerceros!$A$1:$I$495, 6, FALSE), Backend!$B$16:$B$23, 0)), "")</f>
+        <v/>
+      </c>
+      <c r="I15">
+        <f>IF(OR(C15="", G15=""), "", IF(C15&gt;G15, B15, IF(G15&gt;C15, H15, IF(D15&gt;F15, B15, IF(F15&gt;D15, H15, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6460,18 +6517,20 @@
         <v/>
       </c>
       <c r="C16" s="5" t="n"/>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D16" s="38" t="n"/>
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16">
+      <c r="F16" s="38" t="n"/>
+      <c r="G16" s="5" t="n"/>
+      <c r="H16">
         <f>Backend!C13</f>
         <v/>
       </c>
-      <c r="G16">
-        <f>IF(AND(ISNUMBER(C16),ISNUMBER(E16)),IF(C16&gt;E16,B16,F16),"")</f>
+      <c r="I16">
+        <f>IF(OR(C16="", G16=""), "", IF(C16&gt;G16, B16, IF(G16&gt;C16, H16, IF(D16&gt;F16, B16, IF(F16&gt;D16, H16, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6486,18 +6545,20 @@
         <v/>
       </c>
       <c r="C17" s="5" t="n"/>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D17" s="38" t="n"/>
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17">
+      <c r="F17" s="38" t="n"/>
+      <c r="G17" s="5" t="n"/>
+      <c r="H17">
         <f>Backend!C11</f>
         <v/>
       </c>
-      <c r="G17">
-        <f>IF(AND(ISNUMBER(C17),ISNUMBER(E17)),IF(C17&gt;E17,B17,F17),"")</f>
+      <c r="I17">
+        <f>IF(OR(C17="", G17=""), "", IF(C17&gt;G17, B17, IF(G17&gt;C17, H17, IF(D17&gt;F17, B17, IF(F17&gt;D17, H17, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6512,18 +6573,20 @@
         <v/>
       </c>
       <c r="C18" s="5" t="n"/>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D18" s="38" t="n"/>
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18">
-        <f>INDEX(Backend!$C$16:$C$23, MATCH(VLOOKUP(Backend!$D$29, MatrizTerceros!$A$1:$I$495, 3, FALSE), Backend!$B$16:$B$23, 0))</f>
-        <v/>
-      </c>
-      <c r="G18">
-        <f>IF(AND(ISNUMBER(C18),ISNUMBER(E18)),IF(C18&gt;E18,B18,F18),"")</f>
+      <c r="F18" s="38" t="n"/>
+      <c r="G18" s="5" t="n"/>
+      <c r="H18">
+        <f>IFERROR(INDEX(Backend!$C$16:$C$23, MATCH(VLOOKUP(Backend!$D$29, MatrizTerceros!$A$1:$I$495, 3, FALSE), Backend!$B$16:$B$23, 0)), "")</f>
+        <v/>
+      </c>
+      <c r="I18">
+        <f>IF(OR(C18="", G18=""), "", IF(C18&gt;G18, B18, IF(G18&gt;C18, H18, IF(D18&gt;F18, B18, IF(F18&gt;D18, H18, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6538,18 +6601,20 @@
         <v/>
       </c>
       <c r="C19" s="5" t="n"/>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D19" s="38" t="n"/>
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19">
-        <f>INDEX(Backend!$C$16:$C$23, MATCH(VLOOKUP(Backend!$D$29, MatrizTerceros!$A$1:$I$495, 8, FALSE), Backend!$B$16:$B$23, 0))</f>
-        <v/>
-      </c>
-      <c r="G19">
-        <f>IF(AND(ISNUMBER(C19),ISNUMBER(E19)),IF(C19&gt;E19,B19,F19),"")</f>
+      <c r="F19" s="38" t="n"/>
+      <c r="G19" s="5" t="n"/>
+      <c r="H19">
+        <f>IFERROR(INDEX(Backend!$C$16:$C$23, MATCH(VLOOKUP(Backend!$D$29, MatrizTerceros!$A$1:$I$495, 8, FALSE), Backend!$B$16:$B$23, 0)), "")</f>
+        <v/>
+      </c>
+      <c r="I19">
+        <f>IF(OR(C19="", G19=""), "", IF(C19&gt;G19, B19, IF(G19&gt;C19, H19, IF(D19&gt;F19, B19, IF(F19&gt;D19, H19, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6564,18 +6629,20 @@
         <v/>
       </c>
       <c r="C20" s="5" t="n"/>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D20" s="38" t="n"/>
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20">
+      <c r="F20" s="38" t="n"/>
+      <c r="G20" s="5" t="n"/>
+      <c r="H20">
         <f>Backend!C9</f>
         <v/>
       </c>
-      <c r="G20">
-        <f>IF(AND(ISNUMBER(C20),ISNUMBER(E20)),IF(C20&gt;E20,B20,F20),"")</f>
+      <c r="I20">
+        <f>IF(OR(C20="", G20=""), "", IF(C20&gt;G20, B20, IF(G20&gt;C20, H20, IF(D20&gt;F20, B20, IF(F20&gt;D20, H20, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6590,18 +6657,20 @@
         <v/>
       </c>
       <c r="C21" s="5" t="n"/>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D21" s="38" t="n"/>
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E21" s="5" t="n"/>
-      <c r="F21">
+      <c r="F21" s="38" t="n"/>
+      <c r="G21" s="5" t="n"/>
+      <c r="H21">
         <f>Backend!C8</f>
         <v/>
       </c>
-      <c r="G21">
-        <f>IF(AND(ISNUMBER(C21),ISNUMBER(E21)),IF(C21&gt;E21,B21,F21),"")</f>
+      <c r="I21">
+        <f>IF(OR(C21="", G21=""), "", IF(C21&gt;G21, B21, IF(G21&gt;C21, H21, IF(D21&gt;F21, B21, IF(F21&gt;D21, H21, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6619,22 +6688,24 @@
         </is>
       </c>
       <c r="B25">
-        <f>G6</f>
+        <f>I6</f>
         <v/>
       </c>
       <c r="C25" s="5" t="n"/>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="D25" s="38" t="n"/>
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E25" s="5" t="n"/>
-      <c r="F25">
-        <f>G7</f>
-        <v/>
-      </c>
-      <c r="G25">
-        <f>IF(AND(ISNUMBER(C25),ISNUMBER(E25)),IF(C25&gt;E25,B25,F25),"")</f>
+      <c r="F25" s="38" t="n"/>
+      <c r="G25" s="5" t="n"/>
+      <c r="H25">
+        <f>I7</f>
+        <v/>
+      </c>
+      <c r="I25">
+        <f>IF(OR(C25="", G25=""), "", IF(C25&gt;G25, B25, IF(G25&gt;C25, H25, IF(D25&gt;F25, B25, IF(F25&gt;D25, H25, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6645,22 +6716,24 @@
         </is>
       </c>
       <c r="B26">
-        <f>G8</f>
+        <f>I8</f>
         <v/>
       </c>
       <c r="C26" s="5" t="n"/>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="D26" s="38" t="n"/>
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E26" s="5" t="n"/>
-      <c r="F26">
-        <f>G9</f>
-        <v/>
-      </c>
-      <c r="G26">
-        <f>IF(AND(ISNUMBER(C26),ISNUMBER(E26)),IF(C26&gt;E26,B26,F26),"")</f>
+      <c r="F26" s="38" t="n"/>
+      <c r="G26" s="5" t="n"/>
+      <c r="H26">
+        <f>I9</f>
+        <v/>
+      </c>
+      <c r="I26">
+        <f>IF(OR(C26="", G26=""), "", IF(C26&gt;G26, B26, IF(G26&gt;C26, H26, IF(D26&gt;F26, B26, IF(F26&gt;D26, H26, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6671,22 +6744,24 @@
         </is>
       </c>
       <c r="B27">
-        <f>G10</f>
+        <f>I10</f>
         <v/>
       </c>
       <c r="C27" s="5" t="n"/>
-      <c r="D27" s="6" t="inlineStr">
+      <c r="D27" s="38" t="n"/>
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E27" s="5" t="n"/>
-      <c r="F27">
-        <f>G11</f>
-        <v/>
-      </c>
-      <c r="G27">
-        <f>IF(AND(ISNUMBER(C27),ISNUMBER(E27)),IF(C27&gt;E27,B27,F27),"")</f>
+      <c r="F27" s="38" t="n"/>
+      <c r="G27" s="5" t="n"/>
+      <c r="H27">
+        <f>I11</f>
+        <v/>
+      </c>
+      <c r="I27">
+        <f>IF(OR(C27="", G27=""), "", IF(C27&gt;G27, B27, IF(G27&gt;C27, H27, IF(D27&gt;F27, B27, IF(F27&gt;D27, H27, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6697,22 +6772,24 @@
         </is>
       </c>
       <c r="B28">
-        <f>G12</f>
+        <f>I12</f>
         <v/>
       </c>
       <c r="C28" s="5" t="n"/>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="D28" s="38" t="n"/>
+      <c r="E28" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E28" s="5" t="n"/>
-      <c r="F28">
-        <f>G13</f>
-        <v/>
-      </c>
-      <c r="G28">
-        <f>IF(AND(ISNUMBER(C28),ISNUMBER(E28)),IF(C28&gt;E28,B28,F28),"")</f>
+      <c r="F28" s="38" t="n"/>
+      <c r="G28" s="5" t="n"/>
+      <c r="H28">
+        <f>I13</f>
+        <v/>
+      </c>
+      <c r="I28">
+        <f>IF(OR(C28="", G28=""), "", IF(C28&gt;G28, B28, IF(G28&gt;C28, H28, IF(D28&gt;F28, B28, IF(F28&gt;D28, H28, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6723,22 +6800,24 @@
         </is>
       </c>
       <c r="B29">
-        <f>G14</f>
+        <f>I14</f>
         <v/>
       </c>
       <c r="C29" s="5" t="n"/>
-      <c r="D29" s="6" t="inlineStr">
+      <c r="D29" s="38" t="n"/>
+      <c r="E29" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E29" s="5" t="n"/>
-      <c r="F29">
-        <f>G15</f>
-        <v/>
-      </c>
-      <c r="G29">
-        <f>IF(AND(ISNUMBER(C29),ISNUMBER(E29)),IF(C29&gt;E29,B29,F29),"")</f>
+      <c r="F29" s="38" t="n"/>
+      <c r="G29" s="5" t="n"/>
+      <c r="H29">
+        <f>I15</f>
+        <v/>
+      </c>
+      <c r="I29">
+        <f>IF(OR(C29="", G29=""), "", IF(C29&gt;G29, B29, IF(G29&gt;C29, H29, IF(D29&gt;F29, B29, IF(F29&gt;D29, H29, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6749,22 +6828,24 @@
         </is>
       </c>
       <c r="B30">
-        <f>G16</f>
+        <f>I16</f>
         <v/>
       </c>
       <c r="C30" s="5" t="n"/>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="D30" s="38" t="n"/>
+      <c r="E30" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E30" s="5" t="n"/>
-      <c r="F30">
-        <f>G17</f>
-        <v/>
-      </c>
-      <c r="G30">
-        <f>IF(AND(ISNUMBER(C30),ISNUMBER(E30)),IF(C30&gt;E30,B30,F30),"")</f>
+      <c r="F30" s="38" t="n"/>
+      <c r="G30" s="5" t="n"/>
+      <c r="H30">
+        <f>I17</f>
+        <v/>
+      </c>
+      <c r="I30">
+        <f>IF(OR(C30="", G30=""), "", IF(C30&gt;G30, B30, IF(G30&gt;C30, H30, IF(D30&gt;F30, B30, IF(F30&gt;D30, H30, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6775,22 +6856,24 @@
         </is>
       </c>
       <c r="B31">
-        <f>G18</f>
+        <f>I18</f>
         <v/>
       </c>
       <c r="C31" s="5" t="n"/>
-      <c r="D31" s="6" t="inlineStr">
+      <c r="D31" s="38" t="n"/>
+      <c r="E31" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E31" s="5" t="n"/>
-      <c r="F31">
-        <f>G19</f>
-        <v/>
-      </c>
-      <c r="G31">
-        <f>IF(AND(ISNUMBER(C31),ISNUMBER(E31)),IF(C31&gt;E31,B31,F31),"")</f>
+      <c r="F31" s="38" t="n"/>
+      <c r="G31" s="5" t="n"/>
+      <c r="H31">
+        <f>I19</f>
+        <v/>
+      </c>
+      <c r="I31">
+        <f>IF(OR(C31="", G31=""), "", IF(C31&gt;G31, B31, IF(G31&gt;C31, H31, IF(D31&gt;F31, B31, IF(F31&gt;D31, H31, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6801,22 +6884,24 @@
         </is>
       </c>
       <c r="B32">
-        <f>G20</f>
+        <f>I20</f>
         <v/>
       </c>
       <c r="C32" s="5" t="n"/>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="D32" s="38" t="n"/>
+      <c r="E32" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E32" s="5" t="n"/>
-      <c r="F32">
-        <f>G21</f>
-        <v/>
-      </c>
-      <c r="G32">
-        <f>IF(AND(ISNUMBER(C32),ISNUMBER(E32)),IF(C32&gt;E32,B32,F32),"")</f>
+      <c r="F32" s="38" t="n"/>
+      <c r="G32" s="5" t="n"/>
+      <c r="H32">
+        <f>I21</f>
+        <v/>
+      </c>
+      <c r="I32">
+        <f>IF(OR(C32="", G32=""), "", IF(C32&gt;G32, B32, IF(G32&gt;C32, H32, IF(D32&gt;F32, B32, IF(F32&gt;D32, H32, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6824,21 +6909,19 @@
       <c r="A33" s="8" t="n"/>
       <c r="B33" s="8" t="n"/>
       <c r="C33" s="8" t="n"/>
-      <c r="D33" s="8" t="n"/>
       <c r="E33" s="8" t="n"/>
-      <c r="F33" s="8" t="n"/>
       <c r="G33" s="8" t="n"/>
       <c r="H33" s="8" t="n"/>
+      <c r="I33" s="8" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="8" t="n"/>
       <c r="B34" s="8" t="n"/>
       <c r="C34" s="8" t="n"/>
-      <c r="D34" s="8" t="n"/>
       <c r="E34" s="8" t="n"/>
-      <c r="F34" s="8" t="n"/>
       <c r="G34" s="8" t="n"/>
       <c r="H34" s="8" t="n"/>
+      <c r="I34" s="8" t="n"/>
     </row>
     <row r="35" ht="18.75" customHeight="1" s="16">
       <c r="A35" s="28" t="inlineStr">
@@ -6863,29 +6946,24 @@
           <t>Goles</t>
         </is>
       </c>
-      <c r="D36" s="14" t="inlineStr">
+      <c r="E36" s="14" t="inlineStr">
         <is>
           <t>vs</t>
         </is>
       </c>
-      <c r="E36" s="14" t="inlineStr">
+      <c r="G36" s="14" t="inlineStr">
         <is>
           <t>Goles</t>
         </is>
       </c>
-      <c r="F36" s="14" t="inlineStr">
+      <c r="H36" s="14" t="inlineStr">
         <is>
           <t>Equipo B</t>
         </is>
       </c>
-      <c r="G36" s="14" t="inlineStr">
+      <c r="I36" s="14" t="inlineStr">
         <is>
           <t>Clasifica</t>
-        </is>
-      </c>
-      <c r="H36" s="14" t="inlineStr">
-        <is>
-          <t>Estado</t>
         </is>
       </c>
     </row>
@@ -6896,22 +6974,24 @@
         </is>
       </c>
       <c r="B37">
-        <f>G25</f>
+        <f>I25</f>
         <v/>
       </c>
       <c r="C37" s="5" t="n"/>
-      <c r="D37" s="6" t="inlineStr">
+      <c r="D37" s="38" t="n"/>
+      <c r="E37" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E37" s="5" t="n"/>
-      <c r="F37">
-        <f>G26</f>
-        <v/>
-      </c>
-      <c r="G37">
-        <f>IF(AND(ISNUMBER(C37),ISNUMBER(E37)),IF(C37&gt;E37,B37,F37),"")</f>
+      <c r="F37" s="38" t="n"/>
+      <c r="G37" s="5" t="n"/>
+      <c r="H37">
+        <f>I26</f>
+        <v/>
+      </c>
+      <c r="I37">
+        <f>IF(OR(C37="", G37=""), "", IF(C37&gt;G37, B37, IF(G37&gt;C37, H37, IF(D37&gt;F37, B37, IF(F37&gt;D37, H37, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6922,22 +7002,24 @@
         </is>
       </c>
       <c r="B38">
-        <f>G27</f>
+        <f>I27</f>
         <v/>
       </c>
       <c r="C38" s="5" t="n"/>
-      <c r="D38" s="6" t="inlineStr">
+      <c r="D38" s="38" t="n"/>
+      <c r="E38" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E38" s="5" t="n"/>
-      <c r="F38">
-        <f>G28</f>
-        <v/>
-      </c>
-      <c r="G38">
-        <f>IF(AND(ISNUMBER(C38),ISNUMBER(E38)),IF(C38&gt;E38,B38,F38),"")</f>
+      <c r="F38" s="38" t="n"/>
+      <c r="G38" s="5" t="n"/>
+      <c r="H38">
+        <f>I28</f>
+        <v/>
+      </c>
+      <c r="I38">
+        <f>IF(OR(C38="", G38=""), "", IF(C38&gt;G38, B38, IF(G38&gt;C38, H38, IF(D38&gt;F38, B38, IF(F38&gt;D38, H38, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6948,22 +7030,24 @@
         </is>
       </c>
       <c r="B39">
-        <f>G29</f>
+        <f>I29</f>
         <v/>
       </c>
       <c r="C39" s="5" t="n"/>
-      <c r="D39" s="6" t="inlineStr">
+      <c r="D39" s="38" t="n"/>
+      <c r="E39" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E39" s="5" t="n"/>
-      <c r="F39">
-        <f>G30</f>
-        <v/>
-      </c>
-      <c r="G39">
-        <f>IF(AND(ISNUMBER(C39),ISNUMBER(E39)),IF(C39&gt;E39,B39,F39),"")</f>
+      <c r="F39" s="38" t="n"/>
+      <c r="G39" s="5" t="n"/>
+      <c r="H39">
+        <f>I30</f>
+        <v/>
+      </c>
+      <c r="I39">
+        <f>IF(OR(C39="", G39=""), "", IF(C39&gt;G39, B39, IF(G39&gt;C39, H39, IF(D39&gt;F39, B39, IF(F39&gt;D39, H39, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6974,22 +7058,24 @@
         </is>
       </c>
       <c r="B40">
-        <f>G31</f>
+        <f>I31</f>
         <v/>
       </c>
       <c r="C40" s="5" t="n"/>
-      <c r="D40" s="6" t="inlineStr">
+      <c r="D40" s="38" t="n"/>
+      <c r="E40" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E40" s="5" t="n"/>
-      <c r="F40">
-        <f>G32</f>
-        <v/>
-      </c>
-      <c r="G40">
-        <f>IF(AND(ISNUMBER(C40),ISNUMBER(E40)),IF(C40&gt;E40,B40,F40),"")</f>
+      <c r="F40" s="38" t="n"/>
+      <c r="G40" s="5" t="n"/>
+      <c r="H40">
+        <f>I32</f>
+        <v/>
+      </c>
+      <c r="I40">
+        <f>IF(OR(C40="", G40=""), "", IF(C40&gt;G40, B40, IF(G40&gt;C40, H40, IF(D40&gt;F40, B40, IF(F40&gt;D40, H40, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -6997,21 +7083,19 @@
       <c r="A41" s="8" t="n"/>
       <c r="B41" s="8" t="n"/>
       <c r="C41" s="8" t="n"/>
-      <c r="D41" s="8" t="n"/>
       <c r="E41" s="8" t="n"/>
-      <c r="F41" s="8" t="n"/>
       <c r="G41" s="8" t="n"/>
       <c r="H41" s="8" t="n"/>
+      <c r="I41" s="8" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="8" t="n"/>
       <c r="B42" s="8" t="n"/>
       <c r="C42" s="8" t="n"/>
-      <c r="D42" s="8" t="n"/>
       <c r="E42" s="8" t="n"/>
-      <c r="F42" s="8" t="n"/>
       <c r="G42" s="8" t="n"/>
       <c r="H42" s="8" t="n"/>
+      <c r="I42" s="8" t="n"/>
     </row>
     <row r="43" ht="18.75" customHeight="1" s="16">
       <c r="A43" s="28" t="inlineStr">
@@ -7036,29 +7120,24 @@
           <t>Goles</t>
         </is>
       </c>
-      <c r="D44" s="14" t="inlineStr">
+      <c r="E44" s="14" t="inlineStr">
         <is>
           <t>vs</t>
         </is>
       </c>
-      <c r="E44" s="14" t="inlineStr">
+      <c r="G44" s="14" t="inlineStr">
         <is>
           <t>Goles</t>
         </is>
       </c>
-      <c r="F44" s="14" t="inlineStr">
+      <c r="H44" s="14" t="inlineStr">
         <is>
           <t>Equipo B</t>
         </is>
       </c>
-      <c r="G44" s="14" t="inlineStr">
+      <c r="I44" s="14" t="inlineStr">
         <is>
           <t>Clasifica</t>
-        </is>
-      </c>
-      <c r="H44" s="14" t="inlineStr">
-        <is>
-          <t>Estado</t>
         </is>
       </c>
     </row>
@@ -7069,22 +7148,24 @@
         </is>
       </c>
       <c r="B45">
-        <f>G37</f>
+        <f>I37</f>
         <v/>
       </c>
       <c r="C45" s="5" t="n"/>
-      <c r="D45" s="6" t="inlineStr">
+      <c r="D45" s="38" t="n"/>
+      <c r="E45" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E45" s="5" t="n"/>
-      <c r="F45">
-        <f>G38</f>
-        <v/>
-      </c>
-      <c r="G45">
-        <f>IF(AND(ISNUMBER(C45),ISNUMBER(E45)),IF(C45&gt;E45,B45,F45),"")</f>
+      <c r="F45" s="38" t="n"/>
+      <c r="G45" s="5" t="n"/>
+      <c r="H45">
+        <f>I38</f>
+        <v/>
+      </c>
+      <c r="I45">
+        <f>IF(OR(C45="", G45=""), "", IF(C45&gt;G45, B45, IF(G45&gt;C45, H45, IF(D45&gt;F45, B45, IF(F45&gt;D45, H45, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -7095,22 +7176,24 @@
         </is>
       </c>
       <c r="B46">
-        <f>G39</f>
+        <f>I39</f>
         <v/>
       </c>
       <c r="C46" s="5" t="n"/>
-      <c r="D46" s="6" t="inlineStr">
+      <c r="D46" s="38" t="n"/>
+      <c r="E46" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E46" s="5" t="n"/>
-      <c r="F46">
-        <f>G40</f>
-        <v/>
-      </c>
-      <c r="G46">
-        <f>IF(AND(ISNUMBER(C46),ISNUMBER(E46)),IF(C46&gt;E46,B46,F46),"")</f>
+      <c r="F46" s="38" t="n"/>
+      <c r="G46" s="5" t="n"/>
+      <c r="H46">
+        <f>I40</f>
+        <v/>
+      </c>
+      <c r="I46">
+        <f>IF(OR(C46="", G46=""), "", IF(C46&gt;G46, B46, IF(G46&gt;C46, H46, IF(D46&gt;F46, B46, IF(F46&gt;D46, H46, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -7118,21 +7201,19 @@
       <c r="A47" s="8" t="n"/>
       <c r="B47" s="8" t="n"/>
       <c r="C47" s="8" t="n"/>
-      <c r="D47" s="8" t="n"/>
       <c r="E47" s="8" t="n"/>
-      <c r="F47" s="8" t="n"/>
       <c r="G47" s="8" t="n"/>
       <c r="H47" s="8" t="n"/>
+      <c r="I47" s="8" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="8" t="n"/>
       <c r="B48" s="8" t="n"/>
       <c r="C48" s="8" t="n"/>
-      <c r="D48" s="8" t="n"/>
       <c r="E48" s="8" t="n"/>
-      <c r="F48" s="8" t="n"/>
       <c r="G48" s="8" t="n"/>
       <c r="H48" s="8" t="n"/>
+      <c r="I48" s="8" t="n"/>
     </row>
     <row r="49" ht="18.75" customHeight="1" s="16">
       <c r="A49" s="28" t="inlineStr">
@@ -7157,29 +7238,24 @@
           <t>Goles</t>
         </is>
       </c>
-      <c r="D50" s="14" t="inlineStr">
+      <c r="E50" s="14" t="inlineStr">
         <is>
           <t>vs</t>
         </is>
       </c>
-      <c r="E50" s="14" t="inlineStr">
+      <c r="G50" s="14" t="inlineStr">
         <is>
           <t>Goles</t>
         </is>
       </c>
-      <c r="F50" s="14" t="inlineStr">
+      <c r="H50" s="14" t="inlineStr">
         <is>
           <t>Equipo B</t>
         </is>
       </c>
-      <c r="G50" s="14" t="inlineStr">
+      <c r="I50" s="14" t="inlineStr">
         <is>
           <t>Clasifica</t>
-        </is>
-      </c>
-      <c r="H50" s="14" t="inlineStr">
-        <is>
-          <t>Estado</t>
         </is>
       </c>
     </row>
@@ -7190,22 +7266,24 @@
         </is>
       </c>
       <c r="B51">
-        <f>IF(C45&lt;E45,B45,IF(C45&gt;E45,F45,""))</f>
+        <f>IF(OR(C45="", G45=""), "", IF(C45&lt;G45, B45, IF(G45&lt;C45, H45, IF(D45&lt;F45, B45, IF(F45&lt;D45, H45, "")))))</f>
         <v/>
       </c>
       <c r="C51" s="5" t="n"/>
-      <c r="D51" s="6" t="inlineStr">
+      <c r="D51" s="38" t="n"/>
+      <c r="E51" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E51" s="5" t="n"/>
-      <c r="F51">
-        <f>IF(C46&lt;E46,B46,IF(C46&gt;E46,F46,""))</f>
-        <v/>
-      </c>
-      <c r="G51">
-        <f>IF(AND(ISNUMBER(C51),ISNUMBER(E51)),IF(C51&gt;E51,B51,F51),"")</f>
+      <c r="F51" s="38" t="n"/>
+      <c r="G51" s="5" t="n"/>
+      <c r="H51">
+        <f>IF(OR(C46="", G46=""), "", IF(C46&lt;G46, B46, IF(G46&lt;C46, H46, IF(D46&lt;F46, B46, IF(F46&lt;D46, H46, "")))))</f>
+        <v/>
+      </c>
+      <c r="I51">
+        <f>IF(OR(C51="", G51=""), "", IF(C51&gt;G51, B51, IF(G51&gt;C51, H51, IF(D51&gt;F51, B51, IF(F51&gt;D51, H51, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -7213,21 +7291,19 @@
       <c r="A52" s="8" t="n"/>
       <c r="B52" s="8" t="n"/>
       <c r="C52" s="8" t="n"/>
-      <c r="D52" s="8" t="n"/>
       <c r="E52" s="8" t="n"/>
-      <c r="F52" s="8" t="n"/>
       <c r="G52" s="8" t="n"/>
       <c r="H52" s="8" t="n"/>
+      <c r="I52" s="8" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="8" t="n"/>
       <c r="B53" s="8" t="n"/>
       <c r="C53" s="8" t="n"/>
-      <c r="D53" s="8" t="n"/>
       <c r="E53" s="8" t="n"/>
-      <c r="F53" s="8" t="n"/>
       <c r="G53" s="8" t="n"/>
       <c r="H53" s="8" t="n"/>
+      <c r="I53" s="8" t="n"/>
     </row>
     <row r="54" ht="18.75" customHeight="1" s="16">
       <c r="A54" s="28" t="inlineStr">
@@ -7252,29 +7328,24 @@
           <t>Goles</t>
         </is>
       </c>
-      <c r="D55" s="14" t="inlineStr">
+      <c r="E55" s="14" t="inlineStr">
         <is>
           <t>vs</t>
         </is>
       </c>
-      <c r="E55" s="14" t="inlineStr">
+      <c r="G55" s="14" t="inlineStr">
         <is>
           <t>Goles</t>
         </is>
       </c>
-      <c r="F55" s="14" t="inlineStr">
+      <c r="H55" s="14" t="inlineStr">
         <is>
           <t>Equipo B</t>
         </is>
       </c>
-      <c r="G55" s="14" t="inlineStr">
+      <c r="I55" s="14" t="inlineStr">
         <is>
           <t>Clasifica</t>
-        </is>
-      </c>
-      <c r="H55" s="14" t="inlineStr">
-        <is>
-          <t>Estado</t>
         </is>
       </c>
     </row>
@@ -7285,22 +7356,24 @@
         </is>
       </c>
       <c r="B56">
-        <f>G45</f>
+        <f>I45</f>
         <v/>
       </c>
       <c r="C56" s="5" t="n"/>
-      <c r="D56" s="6" t="inlineStr">
+      <c r="D56" s="38" t="n"/>
+      <c r="E56" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E56" s="5" t="n"/>
-      <c r="F56">
-        <f>G46</f>
-        <v/>
-      </c>
-      <c r="G56">
-        <f>IF(AND(ISNUMBER(C56),ISNUMBER(E56)),IF(C56&gt;E56,B56,F56),"")</f>
+      <c r="F56" s="38" t="n"/>
+      <c r="G56" s="5" t="n"/>
+      <c r="H56">
+        <f>I46</f>
+        <v/>
+      </c>
+      <c r="I56">
+        <f>IF(OR(C56="", G56=""), "", IF(C56&gt;G56, B56, IF(G56&gt;C56, H56, IF(D56&gt;F56, B56, IF(F56&gt;D56, H56, "Faltan Penales")))))</f>
         <v/>
       </c>
     </row>
@@ -7308,21 +7381,19 @@
       <c r="A57" s="8" t="n"/>
       <c r="B57" s="8" t="n"/>
       <c r="C57" s="8" t="n"/>
-      <c r="D57" s="8" t="n"/>
       <c r="E57" s="8" t="n"/>
-      <c r="F57" s="8" t="n"/>
       <c r="G57" s="8" t="n"/>
       <c r="H57" s="8" t="n"/>
+      <c r="I57" s="8" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="8" t="n"/>
       <c r="B58" s="8" t="n"/>
       <c r="C58" s="8" t="n"/>
-      <c r="D58" s="8" t="n"/>
       <c r="E58" s="8" t="n"/>
-      <c r="F58" s="8" t="n"/>
       <c r="G58" s="8" t="n"/>
       <c r="H58" s="8" t="n"/>
+      <c r="I58" s="8" t="n"/>
     </row>
     <row r="59" ht="18.75" customHeight="1" s="16">
       <c r="A59" s="28" t="inlineStr">
@@ -7338,12 +7409,11 @@
           <t>CAMPEÓN MUNDIAL 🏆</t>
         </is>
       </c>
-      <c r="F60" s="9">
-        <f>G56</f>
-        <v/>
-      </c>
-      <c r="G60" s="8" t="n"/>
-      <c r="H60" s="8" t="n"/>
+      <c r="H60" s="9">
+        <f>I56</f>
+        <v/>
+      </c>
+      <c r="I60" s="8" t="n"/>
     </row>
     <row r="61" ht="16.5" customHeight="1" s="16">
       <c r="A61" s="8" t="n"/>
@@ -7352,12 +7422,11 @@
           <t>Subcampeón 🥈</t>
         </is>
       </c>
-      <c r="F61" s="9">
-        <f>IF(C56&lt;E56,B56,IF(C56&gt;E56,F56,""))</f>
-        <v/>
-      </c>
-      <c r="G61" s="8" t="n"/>
-      <c r="H61" s="8" t="n"/>
+      <c r="H61" s="9">
+        <f>IF(OR(C56="", G56=""), "", IF(C56&lt;G56, B56, IF(G56&lt;C56, H56, IF(D56&lt;F56, B56, IF(F56&lt;D56, H56, "")))))</f>
+        <v/>
+      </c>
+      <c r="I61" s="8" t="n"/>
     </row>
     <row r="62" ht="16.5" customHeight="1" s="16">
       <c r="A62" s="8" t="n"/>
@@ -7366,26 +7435,25 @@
           <t>Tercer Lugar 🥉</t>
         </is>
       </c>
-      <c r="F62" s="9">
-        <f>G51</f>
-        <v/>
-      </c>
-      <c r="G62" s="8" t="n"/>
-      <c r="H62" s="8" t="n"/>
+      <c r="H62" s="9">
+        <f>I51</f>
+        <v/>
+      </c>
+      <c r="I62" s="8" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="B61:E61"/>
-    <mergeCell ref="A35:H35"/>
-    <mergeCell ref="A59:H59"/>
-    <mergeCell ref="A43:H43"/>
-    <mergeCell ref="A54:H54"/>
-    <mergeCell ref="B62:E62"/>
-    <mergeCell ref="A49:H49"/>
-    <mergeCell ref="A23:H23"/>
-    <mergeCell ref="A1:H2"/>
-    <mergeCell ref="B60:E60"/>
+    <mergeCell ref="A59:I59"/>
+    <mergeCell ref="B62:G62"/>
+    <mergeCell ref="A43:I43"/>
+    <mergeCell ref="A49:I49"/>
+    <mergeCell ref="B60:G60"/>
+    <mergeCell ref="B61:G61"/>
+    <mergeCell ref="A23:I23"/>
+    <mergeCell ref="A1:I2"/>
+    <mergeCell ref="A35:I35"/>
+    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="A54:I54"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add dates to Grupos sheet in template
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_Final_vacia.xlsx
+++ b/Quiniela_Mundial_2026_Final_vacia.xlsx
@@ -8342,6 +8342,7 @@
     <col width="8" customWidth="1" style="28" min="1" max="1"/>
     <col width="16" customWidth="1" style="28" min="3" max="3"/>
     <col width="16" customWidth="1" style="28" min="7" max="7"/>
+    <col width="35" customWidth="1" style="28" min="9" max="9"/>
     <col width="16" customWidth="1" style="28" min="11" max="11"/>
   </cols>
   <sheetData>
@@ -8358,6 +8359,13 @@
       </c>
     </row>
     <row r="2"/>
+    <row r="3">
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Fecha y Hora</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="16.5" customHeight="1" s="28">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -8489,6 +8497,11 @@
         <f>IF(AND(ISNUMBER(D6),ISNUMBER(F6)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Jueves, 11 de junio 2026 - 13:00</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr">
         <is>
           <t>A</t>
@@ -8558,6 +8571,11 @@
         <f>IF(AND(ISNUMBER(D7),ISNUMBER(F7)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Jueves, 11 de junio 2026 - 20:00</t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr">
         <is>
           <t>A</t>
@@ -8627,6 +8645,11 @@
         <f>IF(AND(ISNUMBER(D8),ISNUMBER(F8)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Jueves, 18 de junio 2026 - 19:00</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr">
         <is>
           <t>A</t>
@@ -8696,6 +8719,11 @@
         <f>IF(AND(ISNUMBER(D9),ISNUMBER(F9)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Jueves, 18 de junio 2026 - 10:00</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr">
         <is>
           <t>A</t>
@@ -8765,6 +8793,11 @@
         <f>IF(AND(ISNUMBER(D10),ISNUMBER(F10)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Miércoles, 24 de junio 2026 - 19:00</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="18.75" customHeight="1" s="28">
       <c r="C11" s="4" t="inlineStr">
@@ -8788,6 +8821,11 @@
         <f>IF(AND(ISNUMBER(D11),ISNUMBER(F11)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Miércoles, 24 de junio 2026 - 19:00</t>
+        </is>
+      </c>
       <c r="J11" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO B</t>
@@ -8917,6 +8955,11 @@
         <f>IF(AND(ISNUMBER(D14),ISNUMBER(F14)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Viernes, 12 de junio 2026 - 13:00</t>
+        </is>
+      </c>
       <c r="J14" t="inlineStr">
         <is>
           <t>B</t>
@@ -8986,6 +9029,11 @@
         <f>IF(AND(ISNUMBER(D15),ISNUMBER(F15)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Sábado, 13 de junio 2026 - 13:00</t>
+        </is>
+      </c>
       <c r="J15" t="inlineStr">
         <is>
           <t>B</t>
@@ -9055,6 +9103,11 @@
         <f>IF(AND(ISNUMBER(D16),ISNUMBER(F16)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Jueves, 18 de junio 2026 - 16:00</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18.75" customHeight="1" s="28">
       <c r="C17" s="4" t="inlineStr">
@@ -9078,6 +9131,11 @@
         <f>IF(AND(ISNUMBER(D17),ISNUMBER(F17)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Jueves, 18 de junio 2026 - 13:00</t>
+        </is>
+      </c>
       <c r="J17" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO C</t>
@@ -9106,6 +9164,11 @@
         <f>IF(AND(ISNUMBER(D18),ISNUMBER(F18)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Miércoles, 24 de junio 2026 - 13:00</t>
+        </is>
+      </c>
       <c r="J18" t="inlineStr">
         <is>
           <t>C</t>
@@ -9175,6 +9238,11 @@
         <f>IF(AND(ISNUMBER(D19),ISNUMBER(F19)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Miércoles, 24 de junio 2026 - 13:00</t>
+        </is>
+      </c>
       <c r="J19" t="inlineStr">
         <is>
           <t>C</t>
@@ -9345,6 +9413,11 @@
         <f>IF(AND(ISNUMBER(D22),ISNUMBER(F22)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Sábado, 13 de junio 2026 - 16:00</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="18.75" customHeight="1" s="28">
       <c r="C23" s="4" t="inlineStr">
@@ -9368,6 +9441,11 @@
         <f>IF(AND(ISNUMBER(D23),ISNUMBER(F23)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Sábado, 13 de junio 2026 - 19:00</t>
+        </is>
+      </c>
       <c r="J23" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO D</t>
@@ -9396,6 +9474,11 @@
         <f>IF(AND(ISNUMBER(D24),ISNUMBER(F24)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Viernes, 19 de junio 2026 - 19:00</t>
+        </is>
+      </c>
       <c r="J24" t="inlineStr">
         <is>
           <t>D</t>
@@ -9465,6 +9548,11 @@
         <f>IF(AND(ISNUMBER(D25),ISNUMBER(F25)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Viernes, 19 de junio 2026 - 16:00</t>
+        </is>
+      </c>
       <c r="J25" t="inlineStr">
         <is>
           <t>D</t>
@@ -9534,6 +9622,11 @@
         <f>IF(AND(ISNUMBER(D26),ISNUMBER(F26)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Miércoles, 24 de junio 2026 - 16:00</t>
+        </is>
+      </c>
       <c r="J26" t="inlineStr">
         <is>
           <t>D</t>
@@ -9603,6 +9696,11 @@
         <f>IF(AND(ISNUMBER(D27),ISNUMBER(F27)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Miércoles, 24 de junio 2026 - 16:00</t>
+        </is>
+      </c>
       <c r="J27" t="inlineStr">
         <is>
           <t>D</t>
@@ -9650,6 +9748,7 @@
         <v/>
       </c>
     </row>
+    <row r="28"/>
     <row r="29" ht="18.75" customHeight="1" s="28">
       <c r="A29" s="29" t="inlineStr">
         <is>
@@ -9684,6 +9783,11 @@
         <f>IF(AND(ISNUMBER(D30),ISNUMBER(F30)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Viernes, 12 de junio 2026 - 19:00</t>
+        </is>
+      </c>
       <c r="J30" t="inlineStr">
         <is>
           <t>E</t>
@@ -9753,6 +9857,11 @@
         <f>IF(AND(ISNUMBER(D31),ISNUMBER(F31)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Sábado, 13 de junio 2026 - 22:00</t>
+        </is>
+      </c>
       <c r="J31" t="inlineStr">
         <is>
           <t>E</t>
@@ -9822,6 +9931,11 @@
         <f>IF(AND(ISNUMBER(D32),ISNUMBER(F32)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Viernes, 19 de junio 2026 - 13:00</t>
+        </is>
+      </c>
       <c r="J32" t="inlineStr">
         <is>
           <t>E</t>
@@ -9891,6 +10005,11 @@
         <f>IF(AND(ISNUMBER(D33),ISNUMBER(F33)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Viernes, 19 de junio 2026 - 22:00</t>
+        </is>
+      </c>
       <c r="J33" t="inlineStr">
         <is>
           <t>E</t>
@@ -9960,6 +10079,11 @@
         <f>IF(AND(ISNUMBER(D34),ISNUMBER(F34)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Jueves, 25 de junio 2026 - 20:00</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="18.75" customHeight="1" s="28">
       <c r="C35" s="4" t="inlineStr">
@@ -9983,6 +10107,11 @@
         <f>IF(AND(ISNUMBER(D35),ISNUMBER(F35)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Jueves, 25 de junio 2026 - 20:00</t>
+        </is>
+      </c>
       <c r="J35" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO F</t>
@@ -10181,6 +10310,11 @@
         <f>IF(AND(ISNUMBER(D39),ISNUMBER(F39)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Domingo, 14 de junio 2026 - 17:00</t>
+        </is>
+      </c>
       <c r="J39" t="inlineStr">
         <is>
           <t>F</t>
@@ -10250,6 +10384,11 @@
         <f>IF(AND(ISNUMBER(D40),ISNUMBER(F40)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Sábado, 20 de junio 2026 - 14:00</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="18.75" customHeight="1" s="28">
       <c r="C41" s="4" t="inlineStr">
@@ -10301,6 +10440,11 @@
         <f>IF(AND(ISNUMBER(D42),ISNUMBER(F42)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Jueves, 25 de junio 2026 - 14:00</t>
+        </is>
+      </c>
       <c r="J42" t="inlineStr">
         <is>
           <t>G</t>
@@ -10540,6 +10684,11 @@
         <f>IF(AND(ISNUMBER(D46),ISNUMBER(F46)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Domingo, 14 de junio 2026 - 14:00</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="18.75" customHeight="1" s="28">
       <c r="C47" s="4" t="inlineStr">
@@ -10563,6 +10712,11 @@
         <f>IF(AND(ISNUMBER(D47),ISNUMBER(F47)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Domingo, 14 de junio 2026 - 20:00</t>
+        </is>
+      </c>
       <c r="J47" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO H</t>
@@ -10591,6 +10745,11 @@
         <f>IF(AND(ISNUMBER(D48),ISNUMBER(F48)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Sábado, 20 de junio 2026 - 11:00</t>
+        </is>
+      </c>
       <c r="J48" t="inlineStr">
         <is>
           <t>H</t>
@@ -10660,6 +10819,11 @@
         <f>IF(AND(ISNUMBER(D49),ISNUMBER(F49)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Sábado, 20 de junio 2026 - 22:00</t>
+        </is>
+      </c>
       <c r="J49" t="inlineStr">
         <is>
           <t>H</t>
@@ -10729,6 +10893,11 @@
         <f>IF(AND(ISNUMBER(D50),ISNUMBER(F50)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Jueves, 25 de junio 2026 - 17:00</t>
+        </is>
+      </c>
       <c r="J50" t="inlineStr">
         <is>
           <t>H</t>
@@ -10798,6 +10967,11 @@
         <f>IF(AND(ISNUMBER(D51),ISNUMBER(F51)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Jueves, 25 de junio 2026 - 17:00</t>
+        </is>
+      </c>
       <c r="J51" t="inlineStr">
         <is>
           <t>H</t>
@@ -10845,6 +11019,7 @@
         <v/>
       </c>
     </row>
+    <row r="52"/>
     <row r="53" ht="18.75" customHeight="1" s="28">
       <c r="A53" s="29" t="inlineStr">
         <is>
@@ -10879,6 +11054,11 @@
         <f>IF(AND(ISNUMBER(D54),ISNUMBER(F54)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Lunes, 15 de junio 2026 - 13:00</t>
+        </is>
+      </c>
       <c r="J54" t="inlineStr">
         <is>
           <t>I</t>
@@ -10948,6 +11128,11 @@
         <f>IF(AND(ISNUMBER(D55),ISNUMBER(F55)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Lunes, 15 de junio 2026 - 19:00</t>
+        </is>
+      </c>
       <c r="J55" t="inlineStr">
         <is>
           <t>I</t>
@@ -11017,6 +11202,11 @@
         <f>IF(AND(ISNUMBER(D56),ISNUMBER(F56)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Domingo, 21 de junio 2026 - 13:00</t>
+        </is>
+      </c>
       <c r="J56" t="inlineStr">
         <is>
           <t>I</t>
@@ -11086,6 +11276,11 @@
         <f>IF(AND(ISNUMBER(D57),ISNUMBER(F57)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Domingo, 21 de junio 2026 - 19:00</t>
+        </is>
+      </c>
       <c r="J57" t="inlineStr">
         <is>
           <t>I</t>
@@ -11155,6 +11350,11 @@
         <f>IF(AND(ISNUMBER(D58),ISNUMBER(F58)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Viernes, 26 de junio 2026 - 21:00</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="18.75" customHeight="1" s="28">
       <c r="C59" s="4" t="inlineStr">
@@ -11178,6 +11378,11 @@
         <f>IF(AND(ISNUMBER(D59),ISNUMBER(F59)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Viernes, 26 de junio 2026 - 21:00</t>
+        </is>
+      </c>
       <c r="J59" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO J</t>
@@ -11307,6 +11512,11 @@
         <f>IF(AND(ISNUMBER(D62),ISNUMBER(F62)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Lunes, 15 de junio 2026 - 10:00</t>
+        </is>
+      </c>
       <c r="J62" t="inlineStr">
         <is>
           <t>J</t>
@@ -11376,6 +11586,11 @@
         <f>IF(AND(ISNUMBER(D63),ISNUMBER(F63)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Lunes, 15 de junio 2026 - 16:00</t>
+        </is>
+      </c>
       <c r="J63" t="inlineStr">
         <is>
           <t>J</t>
@@ -11445,6 +11660,11 @@
         <f>IF(AND(ISNUMBER(D64),ISNUMBER(F64)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Domingo, 21 de junio 2026 - 10:00</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="18.75" customHeight="1" s="28">
       <c r="C65" s="4" t="inlineStr">
@@ -11468,6 +11688,11 @@
         <f>IF(AND(ISNUMBER(D65),ISNUMBER(F65)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Domingo, 21 de junio 2026 - 16:00</t>
+        </is>
+      </c>
       <c r="J65" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO K</t>
@@ -11496,6 +11721,11 @@
         <f>IF(AND(ISNUMBER(D66),ISNUMBER(F66)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Viernes, 26 de junio 2026 - 18:00</t>
+        </is>
+      </c>
       <c r="J66" t="inlineStr">
         <is>
           <t>K</t>
@@ -11565,6 +11795,11 @@
         <f>IF(AND(ISNUMBER(D67),ISNUMBER(F67)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Viernes, 26 de junio 2026 - 18:00</t>
+        </is>
+      </c>
       <c r="J67" t="inlineStr">
         <is>
           <t>K</t>
@@ -11735,6 +11970,11 @@
         <f>IF(AND(ISNUMBER(D70),ISNUMBER(F70)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Martes, 16 de junio 2026 - 13:00</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="18.75" customHeight="1" s="28">
       <c r="C71" s="4" t="inlineStr">
@@ -11758,6 +11998,11 @@
         <f>IF(AND(ISNUMBER(D71),ISNUMBER(F71)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Martes, 16 de junio 2026 - 16:00</t>
+        </is>
+      </c>
       <c r="J71" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO L</t>
@@ -11786,6 +12031,11 @@
         <f>IF(AND(ISNUMBER(D72),ISNUMBER(F72)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Lunes, 22 de junio 2026 - 15:00</t>
+        </is>
+      </c>
       <c r="J72" t="inlineStr">
         <is>
           <t>L</t>
@@ -11855,6 +12105,11 @@
         <f>IF(AND(ISNUMBER(D73),ISNUMBER(F73)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Lunes, 22 de junio 2026 - 18:00</t>
+        </is>
+      </c>
       <c r="J73" t="inlineStr">
         <is>
           <t>L</t>
@@ -11924,6 +12179,11 @@
         <f>IF(AND(ISNUMBER(D74),ISNUMBER(F74)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Viernes, 26 de junio 2026 - 13:00</t>
+        </is>
+      </c>
       <c r="J74" t="inlineStr">
         <is>
           <t>L</t>
@@ -11993,6 +12253,11 @@
         <f>IF(AND(ISNUMBER(D75),ISNUMBER(F75)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Viernes, 26 de junio 2026 - 13:00</t>
+        </is>
+      </c>
       <c r="J75" t="inlineStr">
         <is>
           <t>L</t>
@@ -12040,6 +12305,7 @@
         <v/>
       </c>
     </row>
+    <row r="76"/>
     <row r="77" ht="18.75" customHeight="1" s="28">
       <c r="A77" s="29" t="inlineStr">
         <is>
@@ -12069,6 +12335,11 @@
         <f>IF(AND(ISNUMBER(D78),ISNUMBER(F78)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Martes, 16 de junio 2026 - 19:00</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="C79" s="4" t="inlineStr">
@@ -12092,6 +12363,11 @@
         <f>IF(AND(ISNUMBER(D79),ISNUMBER(F79)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Martes, 16 de junio 2026 - 22:00</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="C80" s="4" t="inlineStr">
@@ -12115,6 +12391,11 @@
         <f>IF(AND(ISNUMBER(D80),ISNUMBER(F80)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Lunes, 22 de junio 2026 - 11:00</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="C81" s="4" t="inlineStr">
@@ -12138,6 +12419,11 @@
         <f>IF(AND(ISNUMBER(D81),ISNUMBER(F81)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Lunes, 22 de junio 2026 - 21:00</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="C82" s="4" t="inlineStr">
@@ -12161,6 +12447,11 @@
         <f>IF(AND(ISNUMBER(D82),ISNUMBER(F82)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Sábado, 27 de junio 2026 - 20:00</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="C83" s="4" t="inlineStr">
@@ -12184,7 +12475,13 @@
         <f>IF(AND(ISNUMBER(D83),ISNUMBER(F83)),"Ok","")</f>
         <v/>
       </c>
-    </row>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Sábado, 27 de junio 2026 - 20:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="84"/>
     <row r="85" ht="18.75" customHeight="1" s="28">
       <c r="A85" s="29" t="inlineStr">
         <is>
@@ -12214,6 +12511,11 @@
         <f>IF(AND(ISNUMBER(D86),ISNUMBER(F86)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Miércoles, 17 de junio 2026 - 11:00</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="C87" s="4" t="inlineStr">
@@ -12237,6 +12539,11 @@
         <f>IF(AND(ISNUMBER(D87),ISNUMBER(F87)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Miércoles, 17 de junio 2026 - 20:00</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="C88" s="4" t="inlineStr">
@@ -12260,6 +12567,11 @@
         <f>IF(AND(ISNUMBER(D88),ISNUMBER(F88)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Martes, 23 de junio 2026 - 11:00</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="C89" s="4" t="inlineStr">
@@ -12283,6 +12595,11 @@
         <f>IF(AND(ISNUMBER(D89),ISNUMBER(F89)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Martes, 23 de junio 2026 - 20:00</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="C90" s="4" t="inlineStr">
@@ -12306,6 +12623,11 @@
         <f>IF(AND(ISNUMBER(D90),ISNUMBER(F90)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Sábado, 27 de junio 2026 - 17:30</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="C91" s="4" t="inlineStr">
@@ -12329,7 +12651,13 @@
         <f>IF(AND(ISNUMBER(D91),ISNUMBER(F91)),"Ok","")</f>
         <v/>
       </c>
-    </row>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Sábado, 27 de junio 2026 - 17:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="92"/>
     <row r="93" ht="18.75" customHeight="1" s="28">
       <c r="A93" s="29" t="inlineStr">
         <is>
@@ -12359,6 +12687,11 @@
         <f>IF(AND(ISNUMBER(D94),ISNUMBER(F94)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Miércoles, 17 de junio 2026 - 14:00</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="C95" s="4" t="inlineStr">
@@ -12382,6 +12715,11 @@
         <f>IF(AND(ISNUMBER(D95),ISNUMBER(F95)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Miércoles, 17 de junio 2026 - 17:00</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="C96" s="4" t="inlineStr">
@@ -12405,6 +12743,11 @@
         <f>IF(AND(ISNUMBER(D96),ISNUMBER(F96)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Martes, 23 de junio 2026 - 14:00</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="C97" s="4" t="inlineStr">
@@ -12428,6 +12771,11 @@
         <f>IF(AND(ISNUMBER(D97),ISNUMBER(F97)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Martes, 23 de junio 2026 - 17:00</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="C98" s="4" t="inlineStr">
@@ -12451,6 +12799,11 @@
         <f>IF(AND(ISNUMBER(D98),ISNUMBER(F98)),"Ok","")</f>
         <v/>
       </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Sábado, 27 de junio 2026 - 15:00</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="C99" s="4" t="inlineStr">
@@ -12473,6 +12826,11 @@
       <c r="H99">
         <f>IF(AND(ISNUMBER(D99),ISNUMBER(F99)),"Ok","")</f>
         <v/>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Sábado, 27 de junio 2026 - 15:00</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add dates and locations to Eliminatorias sheet
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_Final_vacia.xlsx
+++ b/Quiniela_Mundial_2026_Final_vacia.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grupos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mejores Terceros" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend" sheetId="4" state="hidden" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eliminatorias" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendario de Juegos" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendario 2" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RankingFIFA" sheetId="8" state="hidden" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MatrizTerceros" sheetId="9" state="hidden" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ranking FIFA" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Grupos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Mejores Terceros" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Backend" sheetId="4" state="hidden" r:id="rId4"/>
+    <sheet name="Eliminatorias" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Calendario de Juegos" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Calendario 2" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="RankingFIFA" sheetId="8" state="hidden" r:id="rId8"/>
+    <sheet name="MatrizTerceros" sheetId="9" state="hidden" r:id="rId9"/>
+    <sheet name="Ranking FIFA" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -147,7 +147,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -211,6 +211,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEAEAEA"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -365,6 +371,7 @@
     <xf numFmtId="0" fontId="17" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -373,7 +380,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -382,182 +389,14 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
   </cellStyles>
-  <dxfs count="12">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD4EDDA"/>
-          <bgColor rgb="FFD4EDDA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD4EDDA"/>
-          <bgColor rgb="FFD4EDDA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD4EDDA"/>
-          <bgColor rgb="FFD4EDDA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD4EDDA"/>
-          <bgColor rgb="FFD4EDDA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD4EDDA"/>
-          <bgColor rgb="FFD4EDDA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD4EDDA"/>
-          <bgColor rgb="FFD4EDDA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD4EDDA"/>
-          <bgColor rgb="FFD4EDDA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD4EDDA"/>
-          <bgColor rgb="FFD4EDDA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD4EDDA"/>
-          <bgColor rgb="FFD4EDDA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD4EDDA"/>
-          <bgColor rgb="FFD4EDDA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD4EDDA"/>
-          <bgColor rgb="FFD4EDDA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD4EDDA"/>
-          <bgColor rgb="FFD4EDDA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <colors/>
 </styleSheet>
 </file>
 
@@ -853,93 +692,93 @@
   <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="148" customWidth="1" style="28" min="1" max="1"/>
-    <col width="75.42578125" customWidth="1" style="28" min="7" max="7"/>
+    <col width="148" customWidth="1" style="29" min="1" max="1"/>
+    <col width="75.42578125" customWidth="1" style="29" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="33.75" customHeight="1" s="28">
+    <row r="1" ht="33.75" customHeight="1" s="29">
       <c r="A1" s="10" t="inlineStr">
         <is>
           <t>QUINIELA MUNDIAL DE FÚTBOL 2026 - 100% AUTOMATIZADA</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="28">
+    <row r="3" ht="16.5" customHeight="1" s="29">
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>La Copa Mundial de la FIFA 26™ tendrá 48 equipos divididos en doce grupos con cuatro equipos cada uno.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="28">
+    <row r="4" ht="16.5" customHeight="1" s="29">
       <c r="A4" s="1" t="n"/>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="28">
+    <row r="5" ht="16.5" customHeight="1" s="29">
       <c r="A5" s="1" t="inlineStr">
         <is>
           <t>Los dos primeros de cada grupo y los ocho mejores terceros avanzarán a los dieciseisavos de final.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="28">
+    <row r="6" ht="16.5" customHeight="1" s="29">
       <c r="A6" s="1" t="n"/>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="28">
+    <row r="7" ht="16.5" customHeight="1" s="29">
       <c r="A7" s="1" t="inlineStr">
         <is>
           <t>Los equipos que lleguen a la final del 19 de julio habrán disputado ocho partidos, uno más que en Catar 2022.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="28">
+    <row r="8" ht="16.5" customHeight="1" s="29">
       <c r="A8" s="1" t="n"/>
     </row>
-    <row r="9" ht="33" customHeight="1" s="28">
+    <row r="9" ht="33" customHeight="1" s="29">
       <c r="A9" s="14" t="inlineStr">
         <is>
           <t>El nuevo esquema establece que los equipos que lleguen a la final, a jugarse el domingo 19 de julio, tendrán que haber atravesado ocho partidos, uno más de los disputados en la última Copa Mundial de la FIFA 2022™, en Catar.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="28">
+    <row r="10" ht="16.5" customHeight="1" s="29">
       <c r="A10" s="1" t="n"/>
     </row>
-    <row r="11" ht="26.25" customHeight="1" s="28">
+    <row r="11" ht="26.25" customHeight="1" s="29">
       <c r="A11" s="10" t="inlineStr">
         <is>
           <t>CÓMO FUNCIONA:</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="28">
+    <row r="13" ht="16.5" customHeight="1" s="29">
       <c r="A13" s="1" t="inlineStr">
         <is>
           <t>1. Pestaña 'Grupos': Ingresa los resultados. Las tablas se calculan en tiempo real.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="28">
+    <row r="14" ht="16.5" customHeight="1" s="29">
       <c r="A14" s="1" t="inlineStr">
         <is>
           <t>2. Pestaña 'Eliminatorias': Al ir llenando, verás cómo los nombres se auto-completan gracias a la corrección del motor.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="28">
+    <row r="15" ht="16.5" customHeight="1" s="29">
       <c r="A15" s="1" t="inlineStr">
         <is>
           <t>3. Puedes empezar a llenar y los líderes de cada grupo aparecerán de inmediato.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="28">
-      <c r="A16" s="34" t="inlineStr">
+    <row r="16" ht="16.5" customHeight="1" s="29">
+      <c r="A16" s="27" t="inlineStr">
         <is>
           <t>4. Guarda tu quiniela con tu nombre y apellido. Ejemplo: Quiniela_Cristiano_Ronaldo.xlsx, Quiniela_Lionel_Messi.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="26.25" customHeight="1" s="28">
+    <row r="17" ht="26.25" customHeight="1" s="29">
       <c r="A17" s="10" t="inlineStr">
         <is>
           <t>Sistema de Puntuación</t>
@@ -949,7 +788,7 @@
     <row r="18">
       <c r="A18" s="7" t="n"/>
     </row>
-    <row r="19" ht="15.75" customHeight="1" s="28">
+    <row r="19" ht="15.75" customHeight="1" s="29">
       <c r="A19" s="15" t="inlineStr">
         <is>
           <t>Fase de Grupos:</t>
@@ -973,7 +812,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="15.75" customHeight="1" s="28">
+    <row r="24" ht="15.75" customHeight="1" s="29">
       <c r="A24" s="15" t="inlineStr">
         <is>
           <t>Fase Eliminatoria:</t>
@@ -1039,7 +878,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="15.75" customHeight="1" s="28">
+    <row r="35" ht="15.75" customHeight="1" s="29">
       <c r="A35" s="15" t="inlineStr">
         <is>
           <t>Podio (Predicciones Finales):</t>
@@ -8339,79 +8178,77 @@
   <dimension ref="A1:T99"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" style="28" min="1" max="1"/>
-    <col width="16" customWidth="1" style="28" min="3" max="3"/>
-    <col width="16" customWidth="1" style="28" min="7" max="7"/>
-    <col width="35" customWidth="1" style="28" min="9" max="9"/>
-    <col width="16" customWidth="1" style="28" min="11" max="11"/>
+    <col width="8" customWidth="1" style="29" min="1" max="1"/>
+    <col width="16" customWidth="1" style="29" min="3" max="3"/>
+    <col width="16" customWidth="1" style="29" min="7" max="7"/>
+    <col width="35" customWidth="1" style="29" min="9" max="9"/>
+    <col width="16" customWidth="1" style="29" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="30" t="inlineStr">
+    <row r="1" ht="15" customHeight="1" s="29">
+      <c r="A1" s="31" t="inlineStr">
         <is>
           <t>PARTIDOS DE GRUPOS</t>
         </is>
       </c>
-      <c r="J1" s="27" t="inlineStr">
+      <c r="J1" s="28" t="inlineStr">
         <is>
           <t>TABLAS DE POSICIONES (AUTOMÁTICAS)</t>
         </is>
       </c>
     </row>
     <row r="2"/>
-    <row r="3">
-      <c r="I3" t="inlineStr">
+    <row r="4" ht="16.5" customHeight="1" s="29">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Grupo</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Equipo 1</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Goles</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Goles</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Equipo 2</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Fecha y Hora</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="16.5" customHeight="1" s="28">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Grupo</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Equipo 1</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Goles</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Goles</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Equipo 2</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>Grupo</t>
-        </is>
-      </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Equipo</t>
@@ -8463,13 +8300,14 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="18.75" customHeight="1" s="28">
-      <c r="A5" s="29" t="inlineStr">
+    <row r="5" ht="18.75" customHeight="1" s="29">
+      <c r="A5" s="30" t="inlineStr">
         <is>
           <t>GRUPO A</t>
         </is>
       </c>
-      <c r="J5" s="29" t="inlineStr">
+      <c r="I5" s="35" t="n"/>
+      <c r="J5" s="30" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO A</t>
         </is>
@@ -8799,7 +8637,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="18.75" customHeight="1" s="28">
+    <row r="11" ht="18.75" customHeight="1" s="29">
       <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Sudáfrica</t>
@@ -8826,7 +8664,7 @@
           <t>Miércoles, 24 de junio 2026 - 19:00</t>
         </is>
       </c>
-      <c r="J11" s="29" t="inlineStr">
+      <c r="J11" s="30" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO B</t>
         </is>
@@ -8880,12 +8718,13 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="18.75" customHeight="1" s="28">
-      <c r="A13" s="29" t="inlineStr">
+    <row r="13" ht="18.75" customHeight="1" s="29">
+      <c r="A13" s="30" t="inlineStr">
         <is>
           <t>GRUPO B</t>
         </is>
       </c>
+      <c r="I13" s="35" t="n"/>
       <c r="J13" t="inlineStr">
         <is>
           <t>B</t>
@@ -9109,7 +8948,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="18.75" customHeight="1" s="28">
+    <row r="17" ht="18.75" customHeight="1" s="29">
       <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Bosnia y Herze.</t>
@@ -9136,7 +8975,7 @@
           <t>Jueves, 18 de junio 2026 - 13:00</t>
         </is>
       </c>
-      <c r="J17" s="29" t="inlineStr">
+      <c r="J17" s="30" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO C</t>
         </is>
@@ -9338,12 +9177,13 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="18.75" customHeight="1" s="28">
-      <c r="A21" s="29" t="inlineStr">
+    <row r="21" ht="18.75" customHeight="1" s="29">
+      <c r="A21" s="30" t="inlineStr">
         <is>
           <t>GRUPO C</t>
         </is>
       </c>
+      <c r="I21" s="35" t="n"/>
       <c r="J21" t="inlineStr">
         <is>
           <t>C</t>
@@ -9419,7 +9259,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="18.75" customHeight="1" s="28">
+    <row r="23" ht="18.75" customHeight="1" s="29">
       <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Haití</t>
@@ -9446,7 +9286,7 @@
           <t>Sábado, 13 de junio 2026 - 19:00</t>
         </is>
       </c>
-      <c r="J23" s="29" t="inlineStr">
+      <c r="J23" s="30" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO D</t>
         </is>
@@ -9748,14 +9588,14 @@
         <v/>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29" ht="18.75" customHeight="1" s="28">
-      <c r="A29" s="29" t="inlineStr">
+    <row r="29" ht="18.75" customHeight="1" s="29">
+      <c r="A29" s="30" t="inlineStr">
         <is>
           <t>GRUPO D</t>
         </is>
       </c>
-      <c r="J29" s="29" t="inlineStr">
+      <c r="I29" s="35" t="n"/>
+      <c r="J29" s="30" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO E</t>
         </is>
@@ -10085,7 +9925,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="18.75" customHeight="1" s="28">
+    <row r="35" ht="18.75" customHeight="1" s="29">
       <c r="C35" s="4" t="inlineStr">
         <is>
           <t>Paraguay</t>
@@ -10112,7 +9952,7 @@
           <t>Jueves, 25 de junio 2026 - 20:00</t>
         </is>
       </c>
-      <c r="J35" s="29" t="inlineStr">
+      <c r="J35" s="30" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO F</t>
         </is>
@@ -10166,12 +10006,13 @@
         <v/>
       </c>
     </row>
-    <row r="37" ht="18.75" customHeight="1" s="28">
-      <c r="A37" s="29" t="inlineStr">
+    <row r="37" ht="18.75" customHeight="1" s="29">
+      <c r="A37" s="30" t="inlineStr">
         <is>
           <t>GRUPO E</t>
         </is>
       </c>
+      <c r="I37" s="35" t="n"/>
       <c r="J37" t="inlineStr">
         <is>
           <t>F</t>
@@ -10395,7 +10236,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="18.75" customHeight="1" s="28">
+    <row r="41" ht="18.75" customHeight="1" s="29">
       <c r="C41" s="4" t="inlineStr">
         <is>
           <t>Curaçao</t>
@@ -10422,7 +10263,7 @@
           <t>Viernes, 19 de junio 2026 - 14:00</t>
         </is>
       </c>
-      <c r="J41" s="29" t="inlineStr">
+      <c r="J41" s="30" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO G</t>
         </is>
@@ -10624,12 +10465,13 @@
         <v/>
       </c>
     </row>
-    <row r="45" ht="18.75" customHeight="1" s="28">
-      <c r="A45" s="29" t="inlineStr">
+    <row r="45" ht="18.75" customHeight="1" s="29">
+      <c r="A45" s="30" t="inlineStr">
         <is>
           <t>GRUPO F</t>
         </is>
       </c>
+      <c r="I45" s="35" t="n"/>
       <c r="J45" t="inlineStr">
         <is>
           <t>G</t>
@@ -10705,7 +10547,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="18.75" customHeight="1" s="28">
+    <row r="47" ht="18.75" customHeight="1" s="29">
       <c r="C47" s="4" t="inlineStr">
         <is>
           <t>Suecia</t>
@@ -10732,7 +10574,7 @@
           <t>Domingo, 14 de junio 2026 - 20:00</t>
         </is>
       </c>
-      <c r="J47" s="29" t="inlineStr">
+      <c r="J47" s="30" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO H</t>
         </is>
@@ -11034,14 +10876,14 @@
         <v/>
       </c>
     </row>
-    <row r="52"/>
-    <row r="53" ht="18.75" customHeight="1" s="28">
-      <c r="A53" s="29" t="inlineStr">
+    <row r="53" ht="18.75" customHeight="1" s="29">
+      <c r="A53" s="30" t="inlineStr">
         <is>
           <t>GRUPO G</t>
         </is>
       </c>
-      <c r="J53" s="29" t="inlineStr">
+      <c r="I53" s="35" t="n"/>
+      <c r="J53" s="30" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO I</t>
         </is>
@@ -11371,7 +11213,7 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="18.75" customHeight="1" s="28">
+    <row r="59" ht="18.75" customHeight="1" s="29">
       <c r="C59" s="4" t="inlineStr">
         <is>
           <t>Egipto</t>
@@ -11398,7 +11240,7 @@
           <t>Viernes, 26 de junio 2026 - 21:00</t>
         </is>
       </c>
-      <c r="J59" s="29" t="inlineStr">
+      <c r="J59" s="30" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO J</t>
         </is>
@@ -11452,12 +11294,13 @@
         <v/>
       </c>
     </row>
-    <row r="61" ht="18.75" customHeight="1" s="28">
-      <c r="A61" s="29" t="inlineStr">
+    <row r="61" ht="18.75" customHeight="1" s="29">
+      <c r="A61" s="30" t="inlineStr">
         <is>
           <t>GRUPO H</t>
         </is>
       </c>
+      <c r="I61" s="35" t="n"/>
       <c r="J61" t="inlineStr">
         <is>
           <t>J</t>
@@ -11681,7 +11524,7 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="18.75" customHeight="1" s="28">
+    <row r="65" ht="18.75" customHeight="1" s="29">
       <c r="C65" s="4" t="inlineStr">
         <is>
           <t>Cabo Verde</t>
@@ -11708,7 +11551,7 @@
           <t>Domingo, 21 de junio 2026 - 16:00</t>
         </is>
       </c>
-      <c r="J65" s="29" t="inlineStr">
+      <c r="J65" s="30" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO K</t>
         </is>
@@ -11910,12 +11753,13 @@
         <v/>
       </c>
     </row>
-    <row r="69" ht="18.75" customHeight="1" s="28">
-      <c r="A69" s="29" t="inlineStr">
+    <row r="69" ht="18.75" customHeight="1" s="29">
+      <c r="A69" s="30" t="inlineStr">
         <is>
           <t>GRUPO I</t>
         </is>
       </c>
+      <c r="I69" s="35" t="n"/>
       <c r="J69" t="inlineStr">
         <is>
           <t>K</t>
@@ -11991,7 +11835,7 @@
         </is>
       </c>
     </row>
-    <row r="71" ht="18.75" customHeight="1" s="28">
+    <row r="71" ht="18.75" customHeight="1" s="29">
       <c r="C71" s="4" t="inlineStr">
         <is>
           <t>Irak</t>
@@ -12018,7 +11862,7 @@
           <t>Martes, 16 de junio 2026 - 16:00</t>
         </is>
       </c>
-      <c r="J71" s="29" t="inlineStr">
+      <c r="J71" s="30" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO L</t>
         </is>
@@ -12320,13 +12164,13 @@
         <v/>
       </c>
     </row>
-    <row r="76"/>
-    <row r="77" ht="18.75" customHeight="1" s="28">
-      <c r="A77" s="29" t="inlineStr">
+    <row r="77" ht="18.75" customHeight="1" s="29">
+      <c r="A77" s="30" t="inlineStr">
         <is>
           <t>GRUPO J</t>
         </is>
       </c>
+      <c r="I77" s="35" t="n"/>
     </row>
     <row r="78">
       <c r="C78" s="4" t="inlineStr">
@@ -12496,13 +12340,13 @@
         </is>
       </c>
     </row>
-    <row r="84"/>
-    <row r="85" ht="18.75" customHeight="1" s="28">
-      <c r="A85" s="29" t="inlineStr">
+    <row r="85" ht="18.75" customHeight="1" s="29">
+      <c r="A85" s="30" t="inlineStr">
         <is>
           <t>GRUPO K</t>
         </is>
       </c>
+      <c r="I85" s="35" t="n"/>
     </row>
     <row r="86">
       <c r="C86" s="4" t="inlineStr">
@@ -12672,13 +12516,13 @@
         </is>
       </c>
     </row>
-    <row r="92"/>
-    <row r="93" ht="18.75" customHeight="1" s="28">
-      <c r="A93" s="29" t="inlineStr">
+    <row r="93" ht="18.75" customHeight="1" s="29">
+      <c r="A93" s="30" t="inlineStr">
         <is>
           <t>GRUPO L</t>
         </is>
       </c>
+      <c r="I93" s="35" t="n"/>
     </row>
     <row r="94">
       <c r="C94" s="4" t="inlineStr">
@@ -12850,9 +12694,8 @@
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="J1:S2"/>
+    <mergeCell ref="J23:T23"/>
     <mergeCell ref="J17:T17"/>
-    <mergeCell ref="J23:T23"/>
     <mergeCell ref="A77:H77"/>
     <mergeCell ref="J29:T29"/>
     <mergeCell ref="J5:T5"/>
@@ -12870,6 +12713,7 @@
     <mergeCell ref="J41:T41"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="A1:H2"/>
+    <mergeCell ref="J1:T2"/>
     <mergeCell ref="A53:H53"/>
     <mergeCell ref="J47:T47"/>
     <mergeCell ref="A29:H29"/>
@@ -12890,22 +12734,22 @@
   <dimension ref="B2:G17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" style="28" min="1" max="1"/>
-    <col width="12" customWidth="1" style="28" min="2" max="3"/>
-    <col width="25" customWidth="1" style="28" min="4" max="4"/>
-    <col width="10" customWidth="1" style="28" min="5" max="6"/>
-    <col width="25" customWidth="1" style="28" min="7" max="7"/>
+    <col width="3" customWidth="1" style="29" min="1" max="1"/>
+    <col width="12" customWidth="1" style="29" min="2" max="3"/>
+    <col width="25" customWidth="1" style="29" min="4" max="4"/>
+    <col width="10" customWidth="1" style="29" min="5" max="6"/>
+    <col width="25" customWidth="1" style="29" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="2">
-      <c r="B2" s="35" t="inlineStr">
+      <c r="B2" s="32" t="inlineStr">
         <is>
           <t>RANKING DE MEJORES TERCEROS LUGARES</t>
         </is>
       </c>
     </row>
     <row r="3"/>
-    <row r="5" ht="16.5" customHeight="1" s="28">
+    <row r="5" ht="16.5" customHeight="1" s="29">
       <c r="B5" s="19" t="inlineStr">
         <is>
           <t>Posición</t>
@@ -12937,7 +12781,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="28">
+    <row r="6" ht="16.5" customHeight="1" s="29">
       <c r="B6" s="20" t="n">
         <v>1</v>
       </c>
@@ -12962,7 +12806,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="28">
+    <row r="7" ht="16.5" customHeight="1" s="29">
       <c r="B7" s="23" t="n">
         <v>2</v>
       </c>
@@ -12987,7 +12831,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="28">
+    <row r="8" ht="16.5" customHeight="1" s="29">
       <c r="B8" s="20" t="n">
         <v>3</v>
       </c>
@@ -13012,7 +12856,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="28">
+    <row r="9" ht="16.5" customHeight="1" s="29">
       <c r="B9" s="23" t="n">
         <v>4</v>
       </c>
@@ -13037,7 +12881,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="28">
+    <row r="10" ht="16.5" customHeight="1" s="29">
       <c r="B10" s="20" t="n">
         <v>5</v>
       </c>
@@ -13062,7 +12906,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="28">
+    <row r="11" ht="16.5" customHeight="1" s="29">
       <c r="B11" s="23" t="n">
         <v>6</v>
       </c>
@@ -13087,7 +12931,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="28">
+    <row r="12" ht="16.5" customHeight="1" s="29">
       <c r="B12" s="20" t="n">
         <v>7</v>
       </c>
@@ -13112,7 +12956,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="28">
+    <row r="13" ht="16.5" customHeight="1" s="29">
       <c r="B13" s="23" t="n">
         <v>8</v>
       </c>
@@ -13137,7 +12981,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="28">
+    <row r="14" ht="16.5" customHeight="1" s="29">
       <c r="B14" s="20" t="n">
         <v>9</v>
       </c>
@@ -13162,7 +13006,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="28">
+    <row r="15" ht="16.5" customHeight="1" s="29">
       <c r="B15" s="23" t="n">
         <v>10</v>
       </c>
@@ -13187,7 +13031,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="28">
+    <row r="16" ht="16.5" customHeight="1" s="29">
       <c r="B16" s="20" t="n">
         <v>11</v>
       </c>
@@ -13212,7 +13056,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="28">
+    <row r="17" ht="16.5" customHeight="1" s="29">
       <c r="B17" s="23" t="n">
         <v>12</v>
       </c>
@@ -13788,32 +13632,40 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:J62"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" style="28" min="2" max="2"/>
-    <col width="6" customWidth="1" style="28" min="3" max="4"/>
-    <col width="3" customWidth="1" style="28" min="5" max="5"/>
-    <col width="6" customWidth="1" style="28" min="6" max="7"/>
-    <col width="18" customWidth="1" style="28" min="8" max="9"/>
+    <col width="20" customWidth="1" style="29" min="2" max="2"/>
+    <col width="6" customWidth="1" style="29" min="3" max="4"/>
+    <col width="3" customWidth="1" style="29" min="5" max="5"/>
+    <col width="6" customWidth="1" style="29" min="6" max="7"/>
+    <col width="18" customWidth="1" style="29" min="8" max="9"/>
+    <col width="45" customWidth="1" style="29" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="30" t="inlineStr">
+      <c r="A1" s="31" t="inlineStr">
         <is>
           <t>FASE FINAL (ELIMINACIÓN DIRECTA)</t>
         </is>
       </c>
     </row>
     <row r="2"/>
-    <row r="4" ht="18.75" customHeight="1" s="28">
-      <c r="A4" s="29" t="inlineStr">
+    <row r="3">
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Fecha y Estadio</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18.75" customHeight="1" s="29">
+      <c r="A4" s="30" t="inlineStr">
         <is>
           <t>DIECISEISAVOS DE FINAL (Ronda de 32)</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="28">
+    <row r="5" ht="16.5" customHeight="1" s="29">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Partido</t>
@@ -13887,6 +13739,11 @@
         <f>IF(OR(C6="", G6=""), "", IF(C6&gt;G6, B6, IF(G6&gt;C6, H6, IF(D6&gt;F6, B6, IF(F6&gt;D6, H6, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Domingo, 28 de junio 2026 - Estadio Los Ángeles</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -13915,6 +13772,11 @@
         <f>IF(OR(C7="", G7=""), "", IF(C7&gt;G7, B7, IF(G7&gt;C7, H7, IF(D7&gt;F7, B7, IF(F7&gt;D7, H7, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Lunes, 29 de junio 2026 - Estadio Boston</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -13943,6 +13805,11 @@
         <f>IF(OR(C8="", G8=""), "", IF(C8&gt;G8, B8, IF(G8&gt;C8, H8, IF(D8&gt;F8, B8, IF(F8&gt;D8, H8, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Lunes, 29 de junio 2026 - Estadio Monterrey</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -13971,6 +13838,11 @@
         <f>IF(OR(C9="", G9=""), "", IF(C9&gt;G9, B9, IF(G9&gt;C9, H9, IF(D9&gt;F9, B9, IF(F9&gt;D9, H9, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Lunes, 29 de junio 2026 - Estadio Houston</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -13999,6 +13871,11 @@
         <f>IF(OR(C10="", G10=""), "", IF(C10&gt;G10, B10, IF(G10&gt;C10, H10, IF(D10&gt;F10, B10, IF(F10&gt;D10, H10, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Martes, 30 de junio 2026 - Estadio Nueva York Nueva Jersey</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -14027,6 +13904,11 @@
         <f>IF(OR(C11="", G11=""), "", IF(C11&gt;G11, B11, IF(G11&gt;C11, H11, IF(D11&gt;F11, B11, IF(F11&gt;D11, H11, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Martes, 30 de junio 2026 - Estadio Dallas</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -14055,6 +13937,11 @@
         <f>IF(OR(C12="", G12=""), "", IF(C12&gt;G12, B12, IF(G12&gt;C12, H12, IF(D12&gt;F12, B12, IF(F12&gt;D12, H12, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Martes, 30 de junio 2026 - Estadio Ciudad de México</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -14083,6 +13970,11 @@
         <f>IF(OR(C13="", G13=""), "", IF(C13&gt;G13, B13, IF(G13&gt;C13, H13, IF(D13&gt;F13, B13, IF(F13&gt;D13, H13, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Miércoles, 1 de julio 2026 - Estadio Atlanta</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -14111,6 +14003,11 @@
         <f>IF(OR(C14="", G14=""), "", IF(C14&gt;G14, B14, IF(G14&gt;C14, H14, IF(D14&gt;F14, B14, IF(F14&gt;D14, H14, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Miércoles, 1 de julio 2026 - Estadio Bahía de San Francisco</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -14139,6 +14036,11 @@
         <f>IF(OR(C15="", G15=""), "", IF(C15&gt;G15, B15, IF(G15&gt;C15, H15, IF(D15&gt;F15, B15, IF(F15&gt;D15, H15, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Miércoles, 1 de julio 2026 - Estadio Seattle</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -14167,6 +14069,11 @@
         <f>IF(OR(C16="", G16=""), "", IF(C16&gt;G16, B16, IF(G16&gt;C16, H16, IF(D16&gt;F16, B16, IF(F16&gt;D16, H16, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Jueves, 2 de julio 2026 - Estadio Toronto</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -14195,6 +14102,11 @@
         <f>IF(OR(C17="", G17=""), "", IF(C17&gt;G17, B17, IF(G17&gt;C17, H17, IF(D17&gt;F17, B17, IF(F17&gt;D17, H17, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Jueves, 2 de julio 2026 - Estadio Los Ángeles</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -14223,6 +14135,11 @@
         <f>IF(OR(C18="", G18=""), "", IF(C18&gt;G18, B18, IF(G18&gt;C18, H18, IF(D18&gt;F18, B18, IF(F18&gt;D18, H18, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Jueves, 2 de julio 2026 - Estadio BC Place Vancouver</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -14251,6 +14168,11 @@
         <f>IF(OR(C19="", G19=""), "", IF(C19&gt;G19, B19, IF(G19&gt;C19, H19, IF(D19&gt;F19, B19, IF(F19&gt;D19, H19, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Viernes, 3 de julio 2026 - Estadio Miami</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -14279,6 +14201,11 @@
         <f>IF(OR(C20="", G20=""), "", IF(C20&gt;G20, B20, IF(G20&gt;C20, H20, IF(D20&gt;F20, B20, IF(F20&gt;D20, H20, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Viernes, 3 de julio 2026 - Estadio Kansas City</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -14307,9 +14234,14 @@
         <f>IF(OR(C21="", G21=""), "", IF(C21&gt;G21, B21, IF(G21&gt;C21, H21, IF(D21&gt;F21, B21, IF(F21&gt;D21, H21, "Faltan Penales")))))</f>
         <v/>
       </c>
-    </row>
-    <row r="23" ht="18.75" customHeight="1" s="28">
-      <c r="A23" s="29" t="inlineStr">
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Viernes, 3 de julio 2026 - Estadio Dallas</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18.75" customHeight="1" s="29">
+      <c r="A23" s="30" t="inlineStr">
         <is>
           <t>OCTAVOS DE FINAL</t>
         </is>
@@ -14342,6 +14274,11 @@
         <f>IF(OR(C25="", G25=""), "", IF(C25&gt;G25, B25, IF(G25&gt;C25, H25, IF(D25&gt;F25, B25, IF(F25&gt;D25, H25, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Sábado, 4 de julio 2026 - Estadio Filadelfia</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -14370,6 +14307,11 @@
         <f>IF(OR(C26="", G26=""), "", IF(C26&gt;G26, B26, IF(G26&gt;C26, H26, IF(D26&gt;F26, B26, IF(F26&gt;D26, H26, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Sábado, 4 de julio 2026 - Estadio Houston</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -14398,6 +14340,11 @@
         <f>IF(OR(C27="", G27=""), "", IF(C27&gt;G27, B27, IF(G27&gt;C27, H27, IF(D27&gt;F27, B27, IF(F27&gt;D27, H27, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Domingo, 5 de julio 2026 - Estadio Nueva York Nueva Jersey</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -14426,6 +14373,11 @@
         <f>IF(OR(C28="", G28=""), "", IF(C28&gt;G28, B28, IF(G28&gt;C28, H28, IF(D28&gt;F28, B28, IF(F28&gt;D28, H28, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Domingo, 5 de julio 2026 - Estadio Ciudad de México</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -14454,6 +14406,11 @@
         <f>IF(OR(C29="", G29=""), "", IF(C29&gt;G29, B29, IF(G29&gt;C29, H29, IF(D29&gt;F29, B29, IF(F29&gt;D29, H29, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Lunes, 6 de julio 2026 - Estadio Dallas</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -14482,6 +14439,11 @@
         <f>IF(OR(C30="", G30=""), "", IF(C30&gt;G30, B30, IF(G30&gt;C30, H30, IF(D30&gt;F30, B30, IF(F30&gt;D30, H30, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Lunes, 6 de julio 2026 - Estadio Seattle</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -14510,6 +14472,11 @@
         <f>IF(OR(C31="", G31=""), "", IF(C31&gt;G31, B31, IF(G31&gt;C31, H31, IF(D31&gt;F31, B31, IF(F31&gt;D31, H31, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Martes, 7 de julio 2026 - Estadio Atlanta</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -14537,6 +14504,11 @@
       <c r="I32">
         <f>IF(OR(C32="", G32=""), "", IF(C32&gt;G32, B32, IF(G32&gt;C32, H32, IF(D32&gt;F32, B32, IF(F32&gt;D32, H32, "Faltan Penales")))))</f>
         <v/>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Martes, 7 de julio 2026 - Estadio BC Place Vancouver</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -14557,14 +14529,14 @@
       <c r="H34" s="8" t="n"/>
       <c r="I34" s="8" t="n"/>
     </row>
-    <row r="35" ht="18.75" customHeight="1" s="28">
-      <c r="A35" s="32" t="inlineStr">
+    <row r="35" ht="18.75" customHeight="1" s="29">
+      <c r="A35" s="33" t="inlineStr">
         <is>
           <t>CUARTOS DE FINAL</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="28">
+    <row r="36" ht="16.5" customHeight="1" s="29">
       <c r="A36" s="2" t="inlineStr">
         <is>
           <t>Partido</t>
@@ -14628,6 +14600,11 @@
         <f>IF(OR(C37="", G37=""), "", IF(C37&gt;G37, B37, IF(G37&gt;C37, H37, IF(D37&gt;F37, B37, IF(F37&gt;D37, H37, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Jueves, 9 de julio 2026 - Estadio Boston</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
@@ -14656,6 +14633,11 @@
         <f>IF(OR(C38="", G38=""), "", IF(C38&gt;G38, B38, IF(G38&gt;C38, H38, IF(D38&gt;F38, B38, IF(F38&gt;D38, H38, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Viernes, 10 de julio 2026 - Estadio Los Ángeles</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
@@ -14684,6 +14666,11 @@
         <f>IF(OR(C39="", G39=""), "", IF(C39&gt;G39, B39, IF(G39&gt;C39, H39, IF(D39&gt;F39, B39, IF(F39&gt;D39, H39, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Sábado, 11 de julio 2026 - Estadio Miami</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
@@ -14711,6 +14698,11 @@
       <c r="I40">
         <f>IF(OR(C40="", G40=""), "", IF(C40&gt;G40, B40, IF(G40&gt;C40, H40, IF(D40&gt;F40, B40, IF(F40&gt;D40, H40, "Faltan Penales")))))</f>
         <v/>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Sábado, 11 de julio 2026 - Estadio Kansas City</t>
+        </is>
       </c>
     </row>
     <row r="41">
@@ -14731,14 +14723,14 @@
       <c r="H42" s="8" t="n"/>
       <c r="I42" s="8" t="n"/>
     </row>
-    <row r="43" ht="18.75" customHeight="1" s="28">
-      <c r="A43" s="32" t="inlineStr">
+    <row r="43" ht="18.75" customHeight="1" s="29">
+      <c r="A43" s="33" t="inlineStr">
         <is>
           <t>SEMIFINALES</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="28">
+    <row r="44" ht="16.5" customHeight="1" s="29">
       <c r="A44" s="2" t="inlineStr">
         <is>
           <t>Partido</t>
@@ -14802,6 +14794,11 @@
         <f>IF(OR(C45="", G45=""), "", IF(C45&gt;G45, B45, IF(G45&gt;C45, H45, IF(D45&gt;F45, B45, IF(F45&gt;D45, H45, "Faltan Penales")))))</f>
         <v/>
       </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Martes, 14 de julio 2026 - Estadio Dallas</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
@@ -14829,6 +14826,11 @@
       <c r="I46">
         <f>IF(OR(C46="", G46=""), "", IF(C46&gt;G46, B46, IF(G46&gt;C46, H46, IF(D46&gt;F46, B46, IF(F46&gt;D46, H46, "Faltan Penales")))))</f>
         <v/>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Miércoles, 15 de julio 2026 - Estadio Atlanta</t>
+        </is>
       </c>
     </row>
     <row r="47">
@@ -14849,14 +14851,14 @@
       <c r="H48" s="8" t="n"/>
       <c r="I48" s="8" t="n"/>
     </row>
-    <row r="49" ht="18.75" customHeight="1" s="28">
-      <c r="A49" s="32" t="inlineStr">
+    <row r="49" ht="18.75" customHeight="1" s="29">
+      <c r="A49" s="33" t="inlineStr">
         <is>
           <t>PARTIDO POR EL TERCER LUGAR</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="28">
+    <row r="50" ht="16.5" customHeight="1" s="29">
       <c r="A50" s="2" t="inlineStr">
         <is>
           <t>Partido</t>
@@ -14919,6 +14921,11 @@
       <c r="I51">
         <f>IF(OR(C51="", G51=""), "", IF(C51&gt;G51, B51, IF(G51&gt;C51, H51, IF(D51&gt;F51, B51, IF(F51&gt;D51, H51, "Faltan Penales")))))</f>
         <v/>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Sábado, 18 de julio 2026 - Estadio Miami</t>
+        </is>
       </c>
     </row>
     <row r="52">
@@ -14939,14 +14946,14 @@
       <c r="H53" s="8" t="n"/>
       <c r="I53" s="8" t="n"/>
     </row>
-    <row r="54" ht="18.75" customHeight="1" s="28">
-      <c r="A54" s="32" t="inlineStr">
+    <row r="54" ht="18.75" customHeight="1" s="29">
+      <c r="A54" s="33" t="inlineStr">
         <is>
           <t>GRAN FINAL</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="16.5" customHeight="1" s="28">
+    <row r="55" ht="16.5" customHeight="1" s="29">
       <c r="A55" s="2" t="inlineStr">
         <is>
           <t>Partido</t>
@@ -15009,6 +15016,11 @@
       <c r="I56">
         <f>IF(OR(C56="", G56=""), "", IF(C56&gt;G56, B56, IF(G56&gt;C56, H56, IF(D56&gt;F56, B56, IF(F56&gt;D56, H56, "Faltan Penales")))))</f>
         <v/>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Domingo, 19 de julio 2026 - Estadio Nueva York Nueva Jersey</t>
+        </is>
       </c>
     </row>
     <row r="57">
@@ -15029,16 +15041,16 @@
       <c r="H58" s="8" t="n"/>
       <c r="I58" s="8" t="n"/>
     </row>
-    <row r="59" ht="18.75" customHeight="1" s="28">
-      <c r="A59" s="32" t="inlineStr">
+    <row r="59" ht="18.75" customHeight="1" s="29">
+      <c r="A59" s="33" t="inlineStr">
         <is>
           <t>PODIO DE HONOR 🏆</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="16.5" customHeight="1" s="28">
+    <row r="60" ht="16.5" customHeight="1" s="29">
       <c r="A60" s="8" t="n"/>
-      <c r="B60" s="33" t="inlineStr">
+      <c r="B60" s="34" t="inlineStr">
         <is>
           <t>CAMPEÓN MUNDIAL 🏆</t>
         </is>
@@ -15049,9 +15061,9 @@
       </c>
       <c r="I60" s="8" t="n"/>
     </row>
-    <row r="61" ht="16.5" customHeight="1" s="28">
+    <row r="61" ht="16.5" customHeight="1" s="29">
       <c r="A61" s="8" t="n"/>
-      <c r="B61" s="33" t="inlineStr">
+      <c r="B61" s="34" t="inlineStr">
         <is>
           <t>Subcampeón 🥈</t>
         </is>
@@ -15062,9 +15074,9 @@
       </c>
       <c r="I61" s="8" t="n"/>
     </row>
-    <row r="62" ht="16.5" customHeight="1" s="28">
+    <row r="62" ht="16.5" customHeight="1" s="29">
       <c r="A62" s="8" t="n"/>
-      <c r="B62" s="33" t="inlineStr">
+      <c r="B62" s="34" t="inlineStr">
         <is>
           <t>Tercer Lugar 🥉</t>
         </is>
@@ -15078,15 +15090,15 @@
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="A59:I59"/>
+    <mergeCell ref="B62:G62"/>
     <mergeCell ref="A43:I43"/>
     <mergeCell ref="A49:I49"/>
     <mergeCell ref="B60:G60"/>
-    <mergeCell ref="A4:I4"/>
     <mergeCell ref="B61:G61"/>
     <mergeCell ref="A23:I23"/>
     <mergeCell ref="A1:I2"/>
     <mergeCell ref="A35:I35"/>
-    <mergeCell ref="B62:G62"/>
+    <mergeCell ref="A4:I4"/>
     <mergeCell ref="A54:I54"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15099,19 +15111,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B183"/>
+  <dimension ref="A1:B183"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="124.28515625" customWidth="1" style="28" min="2" max="2"/>
+    <col width="124.28515625" customWidth="1" style="29" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="2" ht="26.25" customHeight="1" s="28">
+    <row r="1"/>
+    <row r="2" ht="26.25" customHeight="1" s="29">
       <c r="B2" s="10" t="inlineStr">
         <is>
           <t>Fase de grupos: calendario y horarios de la Copa Mundial de la FIFA 2026™</t>
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="B4" s="18" t="inlineStr">
         <is>
@@ -15140,6 +15154,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
@@ -15161,6 +15176,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="B13" t="inlineStr">
         <is>
@@ -15196,6 +15212,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="B19" t="inlineStr">
         <is>
@@ -15231,6 +15248,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="B25" t="inlineStr">
         <is>
@@ -15266,6 +15284,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="B31" t="inlineStr">
         <is>
@@ -15301,6 +15320,7 @@
         </is>
       </c>
     </row>
+    <row r="36"/>
     <row r="37">
       <c r="B37" t="inlineStr">
         <is>
@@ -15336,6 +15356,7 @@
         </is>
       </c>
     </row>
+    <row r="42"/>
     <row r="43">
       <c r="B43" t="inlineStr">
         <is>
@@ -15371,6 +15392,7 @@
         </is>
       </c>
     </row>
+    <row r="48"/>
     <row r="49">
       <c r="B49" t="inlineStr">
         <is>
@@ -15406,6 +15428,7 @@
         </is>
       </c>
     </row>
+    <row r="54"/>
     <row r="55">
       <c r="B55" t="inlineStr">
         <is>
@@ -15441,6 +15464,8 @@
         </is>
       </c>
     </row>
+    <row r="60"/>
+    <row r="61"/>
     <row r="62">
       <c r="B62" t="inlineStr">
         <is>
@@ -15476,6 +15501,7 @@
         </is>
       </c>
     </row>
+    <row r="67"/>
     <row r="68">
       <c r="B68" t="inlineStr">
         <is>
@@ -15511,6 +15537,7 @@
         </is>
       </c>
     </row>
+    <row r="73"/>
     <row r="74">
       <c r="B74" t="inlineStr">
         <is>
@@ -15546,6 +15573,7 @@
         </is>
       </c>
     </row>
+    <row r="79"/>
     <row r="80">
       <c r="B80" t="inlineStr">
         <is>
@@ -15595,6 +15623,7 @@
         </is>
       </c>
     </row>
+    <row r="87"/>
     <row r="88">
       <c r="B88" t="inlineStr">
         <is>
@@ -15644,6 +15673,7 @@
         </is>
       </c>
     </row>
+    <row r="95"/>
     <row r="96">
       <c r="B96" t="inlineStr">
         <is>
@@ -15693,6 +15723,7 @@
         </is>
       </c>
     </row>
+    <row r="103"/>
     <row r="104">
       <c r="B104" t="inlineStr">
         <is>
@@ -15742,6 +15773,7 @@
         </is>
       </c>
     </row>
+    <row r="111"/>
     <row r="112">
       <c r="B112" t="inlineStr">
         <is>
@@ -15749,6 +15781,7 @@
         </is>
       </c>
     </row>
+    <row r="113"/>
     <row r="114">
       <c r="B114" t="inlineStr">
         <is>
@@ -15763,6 +15796,7 @@
         </is>
       </c>
     </row>
+    <row r="116"/>
     <row r="117">
       <c r="B117" t="inlineStr">
         <is>
@@ -15791,6 +15825,7 @@
         </is>
       </c>
     </row>
+    <row r="121"/>
     <row r="122">
       <c r="B122" t="inlineStr">
         <is>
@@ -15819,6 +15854,7 @@
         </is>
       </c>
     </row>
+    <row r="126"/>
     <row r="127">
       <c r="B127" t="inlineStr">
         <is>
@@ -15847,6 +15883,7 @@
         </is>
       </c>
     </row>
+    <row r="131"/>
     <row r="132">
       <c r="B132" t="inlineStr">
         <is>
@@ -15875,6 +15912,7 @@
         </is>
       </c>
     </row>
+    <row r="136"/>
     <row r="137">
       <c r="B137" t="inlineStr">
         <is>
@@ -15903,6 +15941,7 @@
         </is>
       </c>
     </row>
+    <row r="141"/>
     <row r="142">
       <c r="B142" t="inlineStr">
         <is>
@@ -15931,6 +15970,7 @@
         </is>
       </c>
     </row>
+    <row r="146"/>
     <row r="147">
       <c r="B147" t="inlineStr">
         <is>
@@ -15952,6 +15992,7 @@
         </is>
       </c>
     </row>
+    <row r="150"/>
     <row r="151">
       <c r="B151" t="inlineStr">
         <is>
@@ -15973,6 +16014,7 @@
         </is>
       </c>
     </row>
+    <row r="154"/>
     <row r="155">
       <c r="B155" t="inlineStr">
         <is>
@@ -15994,6 +16036,7 @@
         </is>
       </c>
     </row>
+    <row r="158"/>
     <row r="159">
       <c r="B159" t="inlineStr">
         <is>
@@ -16015,6 +16058,7 @@
         </is>
       </c>
     </row>
+    <row r="162"/>
     <row r="163">
       <c r="B163" t="inlineStr">
         <is>
@@ -16029,6 +16073,7 @@
         </is>
       </c>
     </row>
+    <row r="165"/>
     <row r="166">
       <c r="B166" t="inlineStr">
         <is>
@@ -16050,6 +16095,7 @@
         </is>
       </c>
     </row>
+    <row r="169"/>
     <row r="170">
       <c r="B170" t="inlineStr">
         <is>
@@ -16071,6 +16117,7 @@
         </is>
       </c>
     </row>
+    <row r="173"/>
     <row r="174">
       <c r="B174" t="inlineStr">
         <is>
@@ -16085,6 +16132,7 @@
         </is>
       </c>
     </row>
+    <row r="176"/>
     <row r="177">
       <c r="B177" t="inlineStr">
         <is>
@@ -16106,6 +16154,7 @@
         </is>
       </c>
     </row>
+    <row r="180"/>
     <row r="181">
       <c r="B181" t="inlineStr">
         <is>
@@ -16141,24 +16190,24 @@
   <dimension ref="B2:B8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="146" customWidth="1" style="28" min="2" max="2"/>
+    <col width="146" customWidth="1" style="29" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="2" ht="26.25" customHeight="1" s="28">
+    <row r="2" ht="26.25" customHeight="1" s="29">
       <c r="B2" s="10" t="inlineStr">
         <is>
           <t>Link para descargar archvivo ICS del  Calendario Mundial 2026 para Outlook o iPhone:</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="45" customHeight="1" s="28">
+    <row r="3" ht="45" customHeight="1" s="29">
       <c r="B3" s="16" t="inlineStr">
         <is>
           <t>https://calendar.google.com/calendar/ical/611d68120c62daa60625df08296c3333f1416dbeb64241045a3c75dd62f175d8%40group.calendar.google.com/public/basic.ics</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="26.25" customHeight="1" s="28">
+    <row r="6" ht="26.25" customHeight="1" s="29">
       <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Calendario para Google Calendar</t>
@@ -16168,7 +16217,7 @@
     <row r="7">
       <c r="B7" s="17" t="n"/>
     </row>
-    <row r="8" ht="60" customHeight="1" s="28">
+    <row r="8" ht="60" customHeight="1" s="29">
       <c r="B8" s="16" t="inlineStr">
         <is>
           <t>https://calendar.google.com/calendar/u/4?cid=NjExZDY4MTIwYzYyZGFhNjA2MjVkZjA4Mjk2YzMzMzNmMTQxNmRiZWI2NDI0MTA0NWEzYzc1ZGQ2MmYxNzVkOEBncm91cC5jYWxlbmRhci5nb29nbGUuY29t</t>

</xml_diff>